<commit_message>
Them backend Express + ket noi Supabase (Bao cao tong quan va chi tiet)
</commit_message>
<xml_diff>
--- a/public/templates/Report_Template.xlsx
+++ b/public/templates/Report_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trant\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Production Management System\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79134D7E-66D3-498D-92F1-7710FFCE83FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDCD8610-6F3C-4B2E-BAA5-BBC98CCD7CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NHẬT KÝ SẢN XUẤT" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>NHẬT KÝ SẢN XUẤT THEO CA</t>
   </si>
@@ -61,28 +61,7 @@
     <t>Thực hiện (m)</t>
   </si>
   <si>
-    <t>Nguyen Van A</t>
-  </si>
-  <si>
-    <t>Tran Van B</t>
-  </si>
-  <si>
-    <t>Le Van C</t>
-  </si>
-  <si>
-    <t>Đào lò</t>
-  </si>
-  <si>
-    <t>Xén lò</t>
-  </si>
-  <si>
-    <t>Chống đội lò</t>
-  </si>
-  <si>
     <t>Công việc khác</t>
-  </si>
-  <si>
-    <t>Khấu lò</t>
   </si>
   <si>
     <t xml:space="preserve">Giá chống hiện tại </t>
@@ -92,24 +71,6 @@
   </si>
   <si>
     <t>Đơn vị thi công</t>
-  </si>
-  <si>
-    <t>ĐL 1</t>
-  </si>
-  <si>
-    <t>ĐL 2</t>
-  </si>
-  <si>
-    <t>Ổn định</t>
-  </si>
-  <si>
-    <t>Sập lọ cục bộ, đã xử lí</t>
-  </si>
-  <si>
-    <t>KT 1</t>
-  </si>
-  <si>
-    <t>Nguyen Thi A</t>
   </si>
   <si>
     <t>Sản lượng than thực hiện (tấn)</t>
@@ -134,12 +95,6 @@
   </si>
   <si>
     <t>Đường lò</t>
-  </si>
-  <si>
-    <t>DVVT LC 30708 đoạn A6-A8</t>
-  </si>
-  <si>
-    <t>Lò chợ 30705", "XV lò TGVT -340/-275 khu III vỉa 7</t>
   </si>
   <si>
     <t>Thực hiện khấu lò (m)</t>
@@ -270,7 +225,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -349,33 +304,20 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -401,12 +343,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -419,35 +355,36 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,93 +652,86 @@
   <sheetPr>
     <tabColor rgb="FF2E5395"/>
   </sheetPr>
-  <dimension ref="A1:S304"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T304"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.26953125" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" style="24" customWidth="1"/>
+    <col min="3" max="3" width="24.453125" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="12.85546875" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" customWidth="1"/>
-    <col min="16" max="16" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" customWidth="1"/>
-    <col min="18" max="18" width="28.140625" customWidth="1"/>
-    <col min="19" max="19" width="19.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="14.7265625" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" customWidth="1"/>
+    <col min="12" max="12" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="12.81640625" customWidth="1"/>
+    <col min="15" max="15" width="14.453125" customWidth="1"/>
+    <col min="16" max="16" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.7265625" customWidth="1"/>
+    <col min="18" max="18" width="28.1796875" customWidth="1"/>
+    <col min="19" max="19" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-    </row>
-    <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="K2" s="19"/>
-      <c r="L2" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="19"/>
-      <c r="N2" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-    </row>
-    <row r="3" spans="1:19" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="18"/>
+      <c r="S1" s="18"/>
+    </row>
+    <row r="2" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="24"/>
+    </row>
+    <row r="3" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>31</v>
+      <c r="C3" s="13" t="s">
+        <v>18</v>
       </c>
-      <c r="D3" s="16" t="s">
-        <v>17</v>
+      <c r="D3" s="13" t="s">
+        <v>10</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>3</v>
@@ -810,273 +740,133 @@
         <v>4</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>25</v>
+      <c r="H3" s="19" t="s">
+        <v>12</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>26</v>
+      <c r="I3" s="19" t="s">
+        <v>13</v>
       </c>
       <c r="J3" s="20" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
-      <c r="K3" s="10" t="s">
-        <v>28</v>
+      <c r="K3" s="21" t="s">
+        <v>15</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="17" t="s">
-        <v>6</v>
+      <c r="Q3" s="9" t="s">
+        <v>8</v>
       </c>
-      <c r="N3" s="16" t="s">
-        <v>34</v>
+      <c r="R3" s="9" t="s">
+        <v>7</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="R3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="S3" s="11" t="s">
+      <c r="S3" s="9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
-        <v>46204</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="2">
-        <v>32</v>
-      </c>
-      <c r="G4" s="5">
-        <v>3.5</v>
-      </c>
-      <c r="H4" s="5">
-        <v>3.5</v>
-      </c>
-      <c r="I4" s="5">
-        <v>1</v>
-      </c>
-      <c r="J4" s="5">
-        <v>2</v>
-      </c>
-      <c r="K4" s="5">
-        <v>2</v>
-      </c>
-      <c r="L4" s="5">
-        <v>1</v>
-      </c>
-      <c r="M4" s="5">
-        <v>2</v>
-      </c>
-      <c r="N4" s="5">
-        <v>84</v>
-      </c>
-      <c r="O4" s="5">
-        <v>3</v>
-      </c>
-      <c r="P4" s="5">
-        <v>2.8</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>20</v>
-      </c>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A4" s="7"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
-      <c r="S4" s="14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
-        <v>46204</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="2">
-        <v>20</v>
-      </c>
-      <c r="G5" s="5">
-        <v>2</v>
-      </c>
-      <c r="H5" s="5">
-        <v>2</v>
-      </c>
-      <c r="I5" s="5">
-        <v>2</v>
-      </c>
-      <c r="J5" s="5">
-        <v>2</v>
-      </c>
-      <c r="K5" s="5">
-        <v>2</v>
-      </c>
-      <c r="L5" s="5">
-        <v>1</v>
-      </c>
-      <c r="M5" s="5">
-        <v>2</v>
-      </c>
-      <c r="N5" s="5">
-        <v>90</v>
-      </c>
-      <c r="O5" s="5">
-        <v>2</v>
-      </c>
-      <c r="P5" s="5">
-        <v>2</v>
-      </c>
-      <c r="Q5" s="3">
-        <v>20</v>
-      </c>
+      <c r="S4" s="12"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A5" s="7"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="14"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
-        <v>46204</v>
-      </c>
-      <c r="B6" s="1">
-        <v>2</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="2">
-        <v>30</v>
-      </c>
-      <c r="G6" s="5">
-        <v>3.6</v>
-      </c>
-      <c r="H6" s="5">
-        <v>3.2</v>
-      </c>
-      <c r="I6" s="5">
-        <v>1</v>
-      </c>
-      <c r="J6" s="5">
-        <v>3</v>
-      </c>
-      <c r="K6" s="5">
-        <v>2</v>
-      </c>
-      <c r="L6" s="5">
-        <v>1</v>
-      </c>
-      <c r="M6" s="5">
-        <v>2</v>
-      </c>
-      <c r="N6" s="5">
-        <v>93</v>
-      </c>
-      <c r="O6" s="5">
-        <v>3.1</v>
-      </c>
-      <c r="P6" s="5">
-        <v>2.9</v>
-      </c>
-      <c r="Q6" s="3">
-        <v>21</v>
-      </c>
+      <c r="S5" s="12"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="S6" s="6"/>
     </row>
-    <row r="7" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
-        <v>46204</v>
-      </c>
-      <c r="B7" s="1">
-        <v>3</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="2">
-        <v>31</v>
-      </c>
-      <c r="G7" s="5">
-        <v>5.6</v>
-      </c>
-      <c r="H7" s="5">
-        <v>3.6</v>
-      </c>
-      <c r="I7" s="5">
-        <v>1</v>
-      </c>
-      <c r="J7" s="5">
-        <v>4</v>
-      </c>
-      <c r="K7" s="5">
-        <v>2</v>
-      </c>
-      <c r="L7" s="5">
-        <v>1</v>
-      </c>
-      <c r="M7" s="5">
-        <v>1</v>
-      </c>
-      <c r="N7" s="5">
-        <v>93</v>
-      </c>
-      <c r="O7" s="5">
-        <v>3</v>
-      </c>
-      <c r="P7" s="5">
-        <v>3</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>21</v>
-      </c>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
-      <c r="S7" s="14" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S7" s="12"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="7"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="22"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="2"/>
@@ -1094,10 +884,10 @@
       <c r="R8" s="3"/>
       <c r="S8" s="6"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="22"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="2"/>
@@ -1115,10 +905,10 @@
       <c r="R9" s="3"/>
       <c r="S9" s="6"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="22"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="2"/>
@@ -1136,10 +926,10 @@
       <c r="R10" s="3"/>
       <c r="S10" s="6"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="1"/>
-      <c r="C11" s="22"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="2"/>
@@ -1157,10 +947,10 @@
       <c r="R11" s="3"/>
       <c r="S11" s="6"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="22"/>
+      <c r="C12" s="15"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="2"/>
@@ -1178,10 +968,10 @@
       <c r="R12" s="3"/>
       <c r="S12" s="6"/>
     </row>
-    <row r="13" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="22"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="2"/>
@@ -1199,10 +989,10 @@
       <c r="R13" s="3"/>
       <c r="S13" s="6"/>
     </row>
-    <row r="14" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="22"/>
+      <c r="C14" s="15"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="2"/>
@@ -1220,10 +1010,10 @@
       <c r="R14" s="3"/>
       <c r="S14" s="6"/>
     </row>
-    <row r="15" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="22"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="2"/>
@@ -1241,10 +1031,10 @@
       <c r="R15" s="3"/>
       <c r="S15" s="6"/>
     </row>
-    <row r="16" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
       <c r="B16" s="1"/>
-      <c r="C16" s="22"/>
+      <c r="C16" s="15"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="2"/>
@@ -1262,10 +1052,10 @@
       <c r="R16" s="3"/>
       <c r="S16" s="6"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
       <c r="B17" s="1"/>
-      <c r="C17" s="22"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="2"/>
@@ -1283,10 +1073,10 @@
       <c r="R17" s="3"/>
       <c r="S17" s="6"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="22"/>
+      <c r="C18" s="15"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="2"/>
@@ -1304,10 +1094,10 @@
       <c r="R18" s="3"/>
       <c r="S18" s="6"/>
     </row>
-    <row r="19" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="22"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="2"/>
@@ -1325,10 +1115,10 @@
       <c r="R19" s="3"/>
       <c r="S19" s="6"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" s="4"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="22"/>
+      <c r="C20" s="15"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="2"/>
@@ -1346,10 +1136,10 @@
       <c r="R20" s="3"/>
       <c r="S20" s="6"/>
     </row>
-    <row r="21" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="22"/>
+      <c r="C21" s="15"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="2"/>
@@ -1367,10 +1157,10 @@
       <c r="R21" s="3"/>
       <c r="S21" s="6"/>
     </row>
-    <row r="22" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="22"/>
+      <c r="C22" s="15"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="2"/>
@@ -1388,10 +1178,10 @@
       <c r="R22" s="3"/>
       <c r="S22" s="6"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23" s="4"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="22"/>
+      <c r="C23" s="15"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="2"/>
@@ -1409,10 +1199,10 @@
       <c r="R23" s="3"/>
       <c r="S23" s="6"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" s="4"/>
       <c r="B24" s="1"/>
-      <c r="C24" s="22"/>
+      <c r="C24" s="15"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="2"/>
@@ -1430,10 +1220,10 @@
       <c r="R24" s="3"/>
       <c r="S24" s="6"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25" s="4"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="22"/>
+      <c r="C25" s="15"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="2"/>
@@ -1451,10 +1241,10 @@
       <c r="R25" s="3"/>
       <c r="S25" s="6"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26" s="4"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="22"/>
+      <c r="C26" s="15"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="2"/>
@@ -1472,10 +1262,10 @@
       <c r="R26" s="3"/>
       <c r="S26" s="6"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27" s="4"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="22"/>
+      <c r="C27" s="15"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="2"/>
@@ -1493,10 +1283,10 @@
       <c r="R27" s="3"/>
       <c r="S27" s="6"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" s="4"/>
       <c r="B28" s="1"/>
-      <c r="C28" s="22"/>
+      <c r="C28" s="15"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="2"/>
@@ -1514,10 +1304,10 @@
       <c r="R28" s="3"/>
       <c r="S28" s="6"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" s="4"/>
       <c r="B29" s="1"/>
-      <c r="C29" s="22"/>
+      <c r="C29" s="15"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="2"/>
@@ -1535,10 +1325,10 @@
       <c r="R29" s="3"/>
       <c r="S29" s="6"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30" s="4"/>
       <c r="B30" s="1"/>
-      <c r="C30" s="22"/>
+      <c r="C30" s="15"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="2"/>
@@ -1556,10 +1346,10 @@
       <c r="R30" s="3"/>
       <c r="S30" s="6"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31" s="4"/>
       <c r="B31" s="1"/>
-      <c r="C31" s="22"/>
+      <c r="C31" s="15"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="2"/>
@@ -1577,10 +1367,10 @@
       <c r="R31" s="3"/>
       <c r="S31" s="6"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A32" s="4"/>
       <c r="B32" s="1"/>
-      <c r="C32" s="22"/>
+      <c r="C32" s="15"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="2"/>
@@ -1598,10 +1388,10 @@
       <c r="R32" s="3"/>
       <c r="S32" s="6"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A33" s="4"/>
       <c r="B33" s="1"/>
-      <c r="C33" s="22"/>
+      <c r="C33" s="15"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="2"/>
@@ -1619,10 +1409,10 @@
       <c r="R33" s="3"/>
       <c r="S33" s="6"/>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A34" s="4"/>
       <c r="B34" s="1"/>
-      <c r="C34" s="22"/>
+      <c r="C34" s="15"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="2"/>
@@ -1640,10 +1430,10 @@
       <c r="R34" s="3"/>
       <c r="S34" s="6"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A35" s="4"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="22"/>
+      <c r="C35" s="15"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="2"/>
@@ -1661,10 +1451,10 @@
       <c r="R35" s="3"/>
       <c r="S35" s="6"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36" s="4"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="22"/>
+      <c r="C36" s="15"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="2"/>
@@ -1682,10 +1472,10 @@
       <c r="R36" s="3"/>
       <c r="S36" s="6"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A37" s="4"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="22"/>
+      <c r="C37" s="15"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="2"/>
@@ -1703,10 +1493,10 @@
       <c r="R37" s="3"/>
       <c r="S37" s="6"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A38" s="4"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="22"/>
+      <c r="C38" s="15"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="2"/>
@@ -1724,10 +1514,10 @@
       <c r="R38" s="3"/>
       <c r="S38" s="6"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A39" s="4"/>
       <c r="B39" s="1"/>
-      <c r="C39" s="22"/>
+      <c r="C39" s="15"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="2"/>
@@ -1745,10 +1535,10 @@
       <c r="R39" s="3"/>
       <c r="S39" s="6"/>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A40" s="4"/>
       <c r="B40" s="1"/>
-      <c r="C40" s="22"/>
+      <c r="C40" s="15"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="2"/>
@@ -1766,10 +1556,10 @@
       <c r="R40" s="3"/>
       <c r="S40" s="6"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A41" s="4"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="22"/>
+      <c r="C41" s="15"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="2"/>
@@ -1787,10 +1577,10 @@
       <c r="R41" s="3"/>
       <c r="S41" s="6"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A42" s="4"/>
       <c r="B42" s="1"/>
-      <c r="C42" s="22"/>
+      <c r="C42" s="15"/>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
       <c r="F42" s="2"/>
@@ -1808,10 +1598,10 @@
       <c r="R42" s="3"/>
       <c r="S42" s="6"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A43" s="4"/>
       <c r="B43" s="1"/>
-      <c r="C43" s="22"/>
+      <c r="C43" s="15"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="2"/>
@@ -1829,10 +1619,10 @@
       <c r="R43" s="3"/>
       <c r="S43" s="6"/>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A44" s="4"/>
       <c r="B44" s="1"/>
-      <c r="C44" s="22"/>
+      <c r="C44" s="15"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="2"/>
@@ -1850,10 +1640,10 @@
       <c r="R44" s="3"/>
       <c r="S44" s="6"/>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A45" s="4"/>
       <c r="B45" s="1"/>
-      <c r="C45" s="22"/>
+      <c r="C45" s="15"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="2"/>
@@ -1871,10 +1661,10 @@
       <c r="R45" s="3"/>
       <c r="S45" s="6"/>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A46" s="4"/>
       <c r="B46" s="1"/>
-      <c r="C46" s="22"/>
+      <c r="C46" s="15"/>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="2"/>
@@ -1892,10 +1682,10 @@
       <c r="R46" s="3"/>
       <c r="S46" s="6"/>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A47" s="4"/>
       <c r="B47" s="1"/>
-      <c r="C47" s="22"/>
+      <c r="C47" s="15"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="2"/>
@@ -1913,10 +1703,10 @@
       <c r="R47" s="3"/>
       <c r="S47" s="6"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A48" s="4"/>
       <c r="B48" s="1"/>
-      <c r="C48" s="22"/>
+      <c r="C48" s="15"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="2"/>
@@ -1934,10 +1724,10 @@
       <c r="R48" s="3"/>
       <c r="S48" s="6"/>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A49" s="4"/>
       <c r="B49" s="1"/>
-      <c r="C49" s="22"/>
+      <c r="C49" s="15"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="2"/>
@@ -1955,10 +1745,10 @@
       <c r="R49" s="3"/>
       <c r="S49" s="6"/>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A50" s="4"/>
       <c r="B50" s="1"/>
-      <c r="C50" s="22"/>
+      <c r="C50" s="15"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="2"/>
@@ -1976,10 +1766,10 @@
       <c r="R50" s="3"/>
       <c r="S50" s="6"/>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A51" s="4"/>
       <c r="B51" s="1"/>
-      <c r="C51" s="22"/>
+      <c r="C51" s="15"/>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
       <c r="F51" s="2"/>
@@ -1997,10 +1787,10 @@
       <c r="R51" s="3"/>
       <c r="S51" s="6"/>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A52" s="4"/>
       <c r="B52" s="1"/>
-      <c r="C52" s="22"/>
+      <c r="C52" s="15"/>
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
       <c r="F52" s="2"/>
@@ -2018,10 +1808,10 @@
       <c r="R52" s="3"/>
       <c r="S52" s="6"/>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A53" s="4"/>
       <c r="B53" s="1"/>
-      <c r="C53" s="22"/>
+      <c r="C53" s="15"/>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
       <c r="F53" s="2"/>
@@ -2039,10 +1829,10 @@
       <c r="R53" s="3"/>
       <c r="S53" s="6"/>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A54" s="4"/>
       <c r="B54" s="1"/>
-      <c r="C54" s="22"/>
+      <c r="C54" s="15"/>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="2"/>
@@ -2060,10 +1850,10 @@
       <c r="R54" s="3"/>
       <c r="S54" s="6"/>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A55" s="4"/>
       <c r="B55" s="1"/>
-      <c r="C55" s="22"/>
+      <c r="C55" s="15"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="2"/>
@@ -2081,10 +1871,10 @@
       <c r="R55" s="3"/>
       <c r="S55" s="6"/>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A56" s="4"/>
       <c r="B56" s="1"/>
-      <c r="C56" s="22"/>
+      <c r="C56" s="15"/>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
       <c r="F56" s="2"/>
@@ -2102,10 +1892,10 @@
       <c r="R56" s="3"/>
       <c r="S56" s="6"/>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A57" s="4"/>
       <c r="B57" s="1"/>
-      <c r="C57" s="22"/>
+      <c r="C57" s="15"/>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="2"/>
@@ -2123,10 +1913,10 @@
       <c r="R57" s="3"/>
       <c r="S57" s="6"/>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A58" s="4"/>
       <c r="B58" s="1"/>
-      <c r="C58" s="22"/>
+      <c r="C58" s="15"/>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="2"/>
@@ -2144,10 +1934,10 @@
       <c r="R58" s="3"/>
       <c r="S58" s="6"/>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A59" s="4"/>
       <c r="B59" s="1"/>
-      <c r="C59" s="22"/>
+      <c r="C59" s="15"/>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="2"/>
@@ -2165,10 +1955,10 @@
       <c r="R59" s="3"/>
       <c r="S59" s="6"/>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A60" s="4"/>
       <c r="B60" s="1"/>
-      <c r="C60" s="22"/>
+      <c r="C60" s="15"/>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
       <c r="F60" s="2"/>
@@ -2186,10 +1976,10 @@
       <c r="R60" s="3"/>
       <c r="S60" s="6"/>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A61" s="4"/>
       <c r="B61" s="1"/>
-      <c r="C61" s="22"/>
+      <c r="C61" s="15"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="2"/>
@@ -2207,10 +1997,10 @@
       <c r="R61" s="3"/>
       <c r="S61" s="6"/>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A62" s="4"/>
       <c r="B62" s="1"/>
-      <c r="C62" s="22"/>
+      <c r="C62" s="15"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="2"/>
@@ -2228,10 +2018,10 @@
       <c r="R62" s="3"/>
       <c r="S62" s="6"/>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A63" s="4"/>
       <c r="B63" s="1"/>
-      <c r="C63" s="22"/>
+      <c r="C63" s="15"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="2"/>
@@ -2249,10 +2039,10 @@
       <c r="R63" s="3"/>
       <c r="S63" s="6"/>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A64" s="4"/>
       <c r="B64" s="1"/>
-      <c r="C64" s="22"/>
+      <c r="C64" s="15"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="2"/>
@@ -2270,10 +2060,10 @@
       <c r="R64" s="3"/>
       <c r="S64" s="6"/>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A65" s="4"/>
       <c r="B65" s="1"/>
-      <c r="C65" s="22"/>
+      <c r="C65" s="15"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="2"/>
@@ -2291,10 +2081,10 @@
       <c r="R65" s="3"/>
       <c r="S65" s="6"/>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A66" s="4"/>
       <c r="B66" s="1"/>
-      <c r="C66" s="22"/>
+      <c r="C66" s="15"/>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
       <c r="F66" s="2"/>
@@ -2312,10 +2102,10 @@
       <c r="R66" s="3"/>
       <c r="S66" s="6"/>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A67" s="4"/>
       <c r="B67" s="1"/>
-      <c r="C67" s="22"/>
+      <c r="C67" s="15"/>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
       <c r="F67" s="2"/>
@@ -2333,10 +2123,10 @@
       <c r="R67" s="3"/>
       <c r="S67" s="6"/>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A68" s="4"/>
       <c r="B68" s="1"/>
-      <c r="C68" s="22"/>
+      <c r="C68" s="15"/>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
       <c r="F68" s="2"/>
@@ -2354,10 +2144,10 @@
       <c r="R68" s="3"/>
       <c r="S68" s="6"/>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A69" s="4"/>
       <c r="B69" s="1"/>
-      <c r="C69" s="22"/>
+      <c r="C69" s="15"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
       <c r="F69" s="2"/>
@@ -2375,10 +2165,10 @@
       <c r="R69" s="3"/>
       <c r="S69" s="6"/>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A70" s="4"/>
       <c r="B70" s="1"/>
-      <c r="C70" s="22"/>
+      <c r="C70" s="15"/>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
       <c r="F70" s="2"/>
@@ -2396,10 +2186,10 @@
       <c r="R70" s="3"/>
       <c r="S70" s="6"/>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A71" s="4"/>
       <c r="B71" s="1"/>
-      <c r="C71" s="22"/>
+      <c r="C71" s="15"/>
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
       <c r="F71" s="2"/>
@@ -2417,10 +2207,10 @@
       <c r="R71" s="3"/>
       <c r="S71" s="6"/>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A72" s="4"/>
       <c r="B72" s="1"/>
-      <c r="C72" s="22"/>
+      <c r="C72" s="15"/>
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
       <c r="F72" s="2"/>
@@ -2438,10 +2228,10 @@
       <c r="R72" s="3"/>
       <c r="S72" s="6"/>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A73" s="4"/>
       <c r="B73" s="1"/>
-      <c r="C73" s="22"/>
+      <c r="C73" s="15"/>
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
       <c r="F73" s="2"/>
@@ -2459,10 +2249,10 @@
       <c r="R73" s="3"/>
       <c r="S73" s="6"/>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A74" s="4"/>
       <c r="B74" s="1"/>
-      <c r="C74" s="22"/>
+      <c r="C74" s="15"/>
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
       <c r="F74" s="2"/>
@@ -2480,10 +2270,10 @@
       <c r="R74" s="3"/>
       <c r="S74" s="6"/>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A75" s="4"/>
       <c r="B75" s="1"/>
-      <c r="C75" s="22"/>
+      <c r="C75" s="15"/>
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
       <c r="F75" s="2"/>
@@ -2501,10 +2291,10 @@
       <c r="R75" s="3"/>
       <c r="S75" s="6"/>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A76" s="4"/>
       <c r="B76" s="1"/>
-      <c r="C76" s="22"/>
+      <c r="C76" s="15"/>
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" s="2"/>
@@ -2522,10 +2312,10 @@
       <c r="R76" s="3"/>
       <c r="S76" s="6"/>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A77" s="4"/>
       <c r="B77" s="1"/>
-      <c r="C77" s="22"/>
+      <c r="C77" s="15"/>
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
       <c r="F77" s="2"/>
@@ -2543,10 +2333,10 @@
       <c r="R77" s="3"/>
       <c r="S77" s="6"/>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A78" s="4"/>
       <c r="B78" s="1"/>
-      <c r="C78" s="22"/>
+      <c r="C78" s="15"/>
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
       <c r="F78" s="2"/>
@@ -2564,10 +2354,10 @@
       <c r="R78" s="3"/>
       <c r="S78" s="6"/>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A79" s="4"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="22"/>
+      <c r="C79" s="15"/>
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
       <c r="F79" s="2"/>
@@ -2585,10 +2375,10 @@
       <c r="R79" s="3"/>
       <c r="S79" s="6"/>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A80" s="4"/>
       <c r="B80" s="1"/>
-      <c r="C80" s="22"/>
+      <c r="C80" s="15"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="2"/>
@@ -2606,10 +2396,10 @@
       <c r="R80" s="3"/>
       <c r="S80" s="6"/>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A81" s="4"/>
       <c r="B81" s="1"/>
-      <c r="C81" s="22"/>
+      <c r="C81" s="15"/>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
       <c r="F81" s="2"/>
@@ -2627,10 +2417,10 @@
       <c r="R81" s="3"/>
       <c r="S81" s="6"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A82" s="4"/>
       <c r="B82" s="1"/>
-      <c r="C82" s="22"/>
+      <c r="C82" s="15"/>
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
       <c r="F82" s="2"/>
@@ -2648,10 +2438,10 @@
       <c r="R82" s="3"/>
       <c r="S82" s="6"/>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A83" s="4"/>
       <c r="B83" s="1"/>
-      <c r="C83" s="22"/>
+      <c r="C83" s="15"/>
       <c r="D83" s="1"/>
       <c r="E83" s="1"/>
       <c r="F83" s="2"/>
@@ -2669,10 +2459,10 @@
       <c r="R83" s="3"/>
       <c r="S83" s="6"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A84" s="4"/>
       <c r="B84" s="1"/>
-      <c r="C84" s="22"/>
+      <c r="C84" s="15"/>
       <c r="D84" s="1"/>
       <c r="E84" s="1"/>
       <c r="F84" s="2"/>
@@ -2690,10 +2480,10 @@
       <c r="R84" s="3"/>
       <c r="S84" s="6"/>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A85" s="4"/>
       <c r="B85" s="1"/>
-      <c r="C85" s="22"/>
+      <c r="C85" s="15"/>
       <c r="D85" s="1"/>
       <c r="E85" s="1"/>
       <c r="F85" s="2"/>
@@ -2711,10 +2501,10 @@
       <c r="R85" s="3"/>
       <c r="S85" s="6"/>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A86" s="4"/>
       <c r="B86" s="1"/>
-      <c r="C86" s="22"/>
+      <c r="C86" s="15"/>
       <c r="D86" s="1"/>
       <c r="E86" s="1"/>
       <c r="F86" s="2"/>
@@ -2732,10 +2522,10 @@
       <c r="R86" s="3"/>
       <c r="S86" s="6"/>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A87" s="4"/>
       <c r="B87" s="1"/>
-      <c r="C87" s="22"/>
+      <c r="C87" s="15"/>
       <c r="D87" s="1"/>
       <c r="E87" s="1"/>
       <c r="F87" s="2"/>
@@ -2753,10 +2543,10 @@
       <c r="R87" s="3"/>
       <c r="S87" s="6"/>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A88" s="4"/>
       <c r="B88" s="1"/>
-      <c r="C88" s="22"/>
+      <c r="C88" s="15"/>
       <c r="D88" s="1"/>
       <c r="E88" s="1"/>
       <c r="F88" s="2"/>
@@ -2774,10 +2564,10 @@
       <c r="R88" s="3"/>
       <c r="S88" s="6"/>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A89" s="4"/>
       <c r="B89" s="1"/>
-      <c r="C89" s="22"/>
+      <c r="C89" s="15"/>
       <c r="D89" s="1"/>
       <c r="E89" s="1"/>
       <c r="F89" s="2"/>
@@ -2795,10 +2585,10 @@
       <c r="R89" s="3"/>
       <c r="S89" s="6"/>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A90" s="4"/>
       <c r="B90" s="1"/>
-      <c r="C90" s="22"/>
+      <c r="C90" s="15"/>
       <c r="D90" s="1"/>
       <c r="E90" s="1"/>
       <c r="F90" s="2"/>
@@ -2816,10 +2606,10 @@
       <c r="R90" s="3"/>
       <c r="S90" s="6"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A91" s="4"/>
       <c r="B91" s="1"/>
-      <c r="C91" s="22"/>
+      <c r="C91" s="15"/>
       <c r="D91" s="1"/>
       <c r="E91" s="1"/>
       <c r="F91" s="2"/>
@@ -2837,10 +2627,10 @@
       <c r="R91" s="3"/>
       <c r="S91" s="6"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A92" s="4"/>
       <c r="B92" s="1"/>
-      <c r="C92" s="22"/>
+      <c r="C92" s="15"/>
       <c r="D92" s="1"/>
       <c r="E92" s="1"/>
       <c r="F92" s="2"/>
@@ -2858,10 +2648,10 @@
       <c r="R92" s="3"/>
       <c r="S92" s="6"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A93" s="4"/>
       <c r="B93" s="1"/>
-      <c r="C93" s="22"/>
+      <c r="C93" s="15"/>
       <c r="D93" s="1"/>
       <c r="E93" s="1"/>
       <c r="F93" s="2"/>
@@ -2879,10 +2669,10 @@
       <c r="R93" s="3"/>
       <c r="S93" s="6"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A94" s="4"/>
       <c r="B94" s="1"/>
-      <c r="C94" s="22"/>
+      <c r="C94" s="15"/>
       <c r="D94" s="1"/>
       <c r="E94" s="1"/>
       <c r="F94" s="2"/>
@@ -2900,10 +2690,10 @@
       <c r="R94" s="3"/>
       <c r="S94" s="6"/>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A95" s="4"/>
       <c r="B95" s="1"/>
-      <c r="C95" s="22"/>
+      <c r="C95" s="15"/>
       <c r="D95" s="1"/>
       <c r="E95" s="1"/>
       <c r="F95" s="2"/>
@@ -2921,10 +2711,10 @@
       <c r="R95" s="3"/>
       <c r="S95" s="6"/>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A96" s="4"/>
       <c r="B96" s="1"/>
-      <c r="C96" s="22"/>
+      <c r="C96" s="15"/>
       <c r="D96" s="1"/>
       <c r="E96" s="1"/>
       <c r="F96" s="2"/>
@@ -2942,10 +2732,10 @@
       <c r="R96" s="3"/>
       <c r="S96" s="6"/>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A97" s="4"/>
       <c r="B97" s="1"/>
-      <c r="C97" s="22"/>
+      <c r="C97" s="15"/>
       <c r="D97" s="1"/>
       <c r="E97" s="1"/>
       <c r="F97" s="2"/>
@@ -2963,10 +2753,10 @@
       <c r="R97" s="3"/>
       <c r="S97" s="6"/>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A98" s="4"/>
       <c r="B98" s="1"/>
-      <c r="C98" s="22"/>
+      <c r="C98" s="15"/>
       <c r="D98" s="1"/>
       <c r="E98" s="1"/>
       <c r="F98" s="2"/>
@@ -2984,10 +2774,10 @@
       <c r="R98" s="3"/>
       <c r="S98" s="6"/>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A99" s="4"/>
       <c r="B99" s="1"/>
-      <c r="C99" s="22"/>
+      <c r="C99" s="15"/>
       <c r="D99" s="1"/>
       <c r="E99" s="1"/>
       <c r="F99" s="2"/>
@@ -3005,10 +2795,10 @@
       <c r="R99" s="3"/>
       <c r="S99" s="6"/>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A100" s="4"/>
       <c r="B100" s="1"/>
-      <c r="C100" s="22"/>
+      <c r="C100" s="15"/>
       <c r="D100" s="1"/>
       <c r="E100" s="1"/>
       <c r="F100" s="2"/>
@@ -3026,10 +2816,10 @@
       <c r="R100" s="3"/>
       <c r="S100" s="6"/>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A101" s="4"/>
       <c r="B101" s="1"/>
-      <c r="C101" s="22"/>
+      <c r="C101" s="15"/>
       <c r="D101" s="1"/>
       <c r="E101" s="1"/>
       <c r="F101" s="2"/>
@@ -3047,10 +2837,10 @@
       <c r="R101" s="3"/>
       <c r="S101" s="6"/>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A102" s="4"/>
       <c r="B102" s="1"/>
-      <c r="C102" s="22"/>
+      <c r="C102" s="15"/>
       <c r="D102" s="1"/>
       <c r="E102" s="1"/>
       <c r="F102" s="2"/>
@@ -3068,10 +2858,10 @@
       <c r="R102" s="3"/>
       <c r="S102" s="6"/>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A103" s="4"/>
       <c r="B103" s="1"/>
-      <c r="C103" s="22"/>
+      <c r="C103" s="15"/>
       <c r="D103" s="1"/>
       <c r="E103" s="1"/>
       <c r="F103" s="2"/>
@@ -3089,10 +2879,10 @@
       <c r="R103" s="3"/>
       <c r="S103" s="6"/>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A104" s="4"/>
       <c r="B104" s="1"/>
-      <c r="C104" s="22"/>
+      <c r="C104" s="15"/>
       <c r="D104" s="1"/>
       <c r="E104" s="1"/>
       <c r="F104" s="2"/>
@@ -3110,10 +2900,10 @@
       <c r="R104" s="3"/>
       <c r="S104" s="6"/>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A105" s="4"/>
       <c r="B105" s="1"/>
-      <c r="C105" s="22"/>
+      <c r="C105" s="15"/>
       <c r="D105" s="1"/>
       <c r="E105" s="1"/>
       <c r="F105" s="2"/>
@@ -3131,10 +2921,10 @@
       <c r="R105" s="3"/>
       <c r="S105" s="6"/>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A106" s="4"/>
       <c r="B106" s="1"/>
-      <c r="C106" s="22"/>
+      <c r="C106" s="15"/>
       <c r="D106" s="1"/>
       <c r="E106" s="1"/>
       <c r="F106" s="2"/>
@@ -3152,10 +2942,10 @@
       <c r="R106" s="3"/>
       <c r="S106" s="6"/>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A107" s="4"/>
       <c r="B107" s="1"/>
-      <c r="C107" s="22"/>
+      <c r="C107" s="15"/>
       <c r="D107" s="1"/>
       <c r="E107" s="1"/>
       <c r="F107" s="2"/>
@@ -3173,10 +2963,10 @@
       <c r="R107" s="3"/>
       <c r="S107" s="6"/>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A108" s="4"/>
       <c r="B108" s="1"/>
-      <c r="C108" s="22"/>
+      <c r="C108" s="15"/>
       <c r="D108" s="1"/>
       <c r="E108" s="1"/>
       <c r="F108" s="2"/>
@@ -3194,10 +2984,10 @@
       <c r="R108" s="3"/>
       <c r="S108" s="6"/>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A109" s="4"/>
       <c r="B109" s="1"/>
-      <c r="C109" s="22"/>
+      <c r="C109" s="15"/>
       <c r="D109" s="1"/>
       <c r="E109" s="1"/>
       <c r="F109" s="2"/>
@@ -3215,10 +3005,10 @@
       <c r="R109" s="3"/>
       <c r="S109" s="6"/>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A110" s="4"/>
       <c r="B110" s="1"/>
-      <c r="C110" s="22"/>
+      <c r="C110" s="15"/>
       <c r="D110" s="1"/>
       <c r="E110" s="1"/>
       <c r="F110" s="2"/>
@@ -3236,10 +3026,10 @@
       <c r="R110" s="3"/>
       <c r="S110" s="6"/>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A111" s="4"/>
       <c r="B111" s="1"/>
-      <c r="C111" s="22"/>
+      <c r="C111" s="15"/>
       <c r="D111" s="1"/>
       <c r="E111" s="1"/>
       <c r="F111" s="2"/>
@@ -3257,10 +3047,10 @@
       <c r="R111" s="3"/>
       <c r="S111" s="6"/>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A112" s="4"/>
       <c r="B112" s="1"/>
-      <c r="C112" s="22"/>
+      <c r="C112" s="15"/>
       <c r="D112" s="1"/>
       <c r="E112" s="1"/>
       <c r="F112" s="2"/>
@@ -3278,10 +3068,10 @@
       <c r="R112" s="3"/>
       <c r="S112" s="6"/>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A113" s="4"/>
       <c r="B113" s="1"/>
-      <c r="C113" s="22"/>
+      <c r="C113" s="15"/>
       <c r="D113" s="1"/>
       <c r="E113" s="1"/>
       <c r="F113" s="2"/>
@@ -3299,10 +3089,10 @@
       <c r="R113" s="3"/>
       <c r="S113" s="6"/>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A114" s="4"/>
       <c r="B114" s="1"/>
-      <c r="C114" s="22"/>
+      <c r="C114" s="15"/>
       <c r="D114" s="1"/>
       <c r="E114" s="1"/>
       <c r="F114" s="2"/>
@@ -3320,10 +3110,10 @@
       <c r="R114" s="3"/>
       <c r="S114" s="6"/>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A115" s="4"/>
       <c r="B115" s="1"/>
-      <c r="C115" s="22"/>
+      <c r="C115" s="15"/>
       <c r="D115" s="1"/>
       <c r="E115" s="1"/>
       <c r="F115" s="2"/>
@@ -3341,10 +3131,10 @@
       <c r="R115" s="3"/>
       <c r="S115" s="6"/>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A116" s="4"/>
       <c r="B116" s="1"/>
-      <c r="C116" s="22"/>
+      <c r="C116" s="15"/>
       <c r="D116" s="1"/>
       <c r="E116" s="1"/>
       <c r="F116" s="2"/>
@@ -3362,10 +3152,10 @@
       <c r="R116" s="3"/>
       <c r="S116" s="6"/>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A117" s="4"/>
       <c r="B117" s="1"/>
-      <c r="C117" s="22"/>
+      <c r="C117" s="15"/>
       <c r="D117" s="1"/>
       <c r="E117" s="1"/>
       <c r="F117" s="2"/>
@@ -3383,10 +3173,10 @@
       <c r="R117" s="3"/>
       <c r="S117" s="6"/>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A118" s="4"/>
       <c r="B118" s="1"/>
-      <c r="C118" s="22"/>
+      <c r="C118" s="15"/>
       <c r="D118" s="1"/>
       <c r="E118" s="1"/>
       <c r="F118" s="2"/>
@@ -3404,10 +3194,10 @@
       <c r="R118" s="3"/>
       <c r="S118" s="6"/>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A119" s="4"/>
       <c r="B119" s="1"/>
-      <c r="C119" s="22"/>
+      <c r="C119" s="15"/>
       <c r="D119" s="1"/>
       <c r="E119" s="1"/>
       <c r="F119" s="2"/>
@@ -3425,10 +3215,10 @@
       <c r="R119" s="3"/>
       <c r="S119" s="6"/>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A120" s="4"/>
       <c r="B120" s="1"/>
-      <c r="C120" s="22"/>
+      <c r="C120" s="15"/>
       <c r="D120" s="1"/>
       <c r="E120" s="1"/>
       <c r="F120" s="2"/>
@@ -3446,10 +3236,10 @@
       <c r="R120" s="3"/>
       <c r="S120" s="6"/>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A121" s="4"/>
       <c r="B121" s="1"/>
-      <c r="C121" s="22"/>
+      <c r="C121" s="15"/>
       <c r="D121" s="1"/>
       <c r="E121" s="1"/>
       <c r="F121" s="2"/>
@@ -3467,10 +3257,10 @@
       <c r="R121" s="3"/>
       <c r="S121" s="6"/>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A122" s="4"/>
       <c r="B122" s="1"/>
-      <c r="C122" s="22"/>
+      <c r="C122" s="15"/>
       <c r="D122" s="1"/>
       <c r="E122" s="1"/>
       <c r="F122" s="2"/>
@@ -3488,10 +3278,10 @@
       <c r="R122" s="3"/>
       <c r="S122" s="6"/>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A123" s="4"/>
       <c r="B123" s="1"/>
-      <c r="C123" s="22"/>
+      <c r="C123" s="15"/>
       <c r="D123" s="1"/>
       <c r="E123" s="1"/>
       <c r="F123" s="2"/>
@@ -3509,10 +3299,10 @@
       <c r="R123" s="3"/>
       <c r="S123" s="6"/>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A124" s="4"/>
       <c r="B124" s="1"/>
-      <c r="C124" s="22"/>
+      <c r="C124" s="15"/>
       <c r="D124" s="1"/>
       <c r="E124" s="1"/>
       <c r="F124" s="2"/>
@@ -3530,10 +3320,10 @@
       <c r="R124" s="3"/>
       <c r="S124" s="6"/>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A125" s="4"/>
       <c r="B125" s="1"/>
-      <c r="C125" s="22"/>
+      <c r="C125" s="15"/>
       <c r="D125" s="1"/>
       <c r="E125" s="1"/>
       <c r="F125" s="2"/>
@@ -3551,10 +3341,10 @@
       <c r="R125" s="3"/>
       <c r="S125" s="6"/>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A126" s="4"/>
       <c r="B126" s="1"/>
-      <c r="C126" s="22"/>
+      <c r="C126" s="15"/>
       <c r="D126" s="1"/>
       <c r="E126" s="1"/>
       <c r="F126" s="2"/>
@@ -3572,10 +3362,10 @@
       <c r="R126" s="3"/>
       <c r="S126" s="6"/>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A127" s="4"/>
       <c r="B127" s="1"/>
-      <c r="C127" s="22"/>
+      <c r="C127" s="15"/>
       <c r="D127" s="1"/>
       <c r="E127" s="1"/>
       <c r="F127" s="2"/>
@@ -3593,10 +3383,10 @@
       <c r="R127" s="3"/>
       <c r="S127" s="6"/>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A128" s="4"/>
       <c r="B128" s="1"/>
-      <c r="C128" s="22"/>
+      <c r="C128" s="15"/>
       <c r="D128" s="1"/>
       <c r="E128" s="1"/>
       <c r="F128" s="2"/>
@@ -3614,10 +3404,10 @@
       <c r="R128" s="3"/>
       <c r="S128" s="6"/>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A129" s="4"/>
       <c r="B129" s="1"/>
-      <c r="C129" s="22"/>
+      <c r="C129" s="15"/>
       <c r="D129" s="1"/>
       <c r="E129" s="1"/>
       <c r="F129" s="2"/>
@@ -3635,10 +3425,10 @@
       <c r="R129" s="3"/>
       <c r="S129" s="6"/>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A130" s="4"/>
       <c r="B130" s="1"/>
-      <c r="C130" s="22"/>
+      <c r="C130" s="15"/>
       <c r="D130" s="1"/>
       <c r="E130" s="1"/>
       <c r="F130" s="2"/>
@@ -3656,10 +3446,10 @@
       <c r="R130" s="3"/>
       <c r="S130" s="6"/>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A131" s="4"/>
       <c r="B131" s="1"/>
-      <c r="C131" s="22"/>
+      <c r="C131" s="15"/>
       <c r="D131" s="1"/>
       <c r="E131" s="1"/>
       <c r="F131" s="2"/>
@@ -3677,10 +3467,10 @@
       <c r="R131" s="3"/>
       <c r="S131" s="6"/>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A132" s="4"/>
       <c r="B132" s="1"/>
-      <c r="C132" s="22"/>
+      <c r="C132" s="15"/>
       <c r="D132" s="1"/>
       <c r="E132" s="1"/>
       <c r="F132" s="2"/>
@@ -3698,10 +3488,10 @@
       <c r="R132" s="3"/>
       <c r="S132" s="6"/>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A133" s="4"/>
       <c r="B133" s="1"/>
-      <c r="C133" s="22"/>
+      <c r="C133" s="15"/>
       <c r="D133" s="1"/>
       <c r="E133" s="1"/>
       <c r="F133" s="2"/>
@@ -3719,10 +3509,10 @@
       <c r="R133" s="3"/>
       <c r="S133" s="6"/>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A134" s="4"/>
       <c r="B134" s="1"/>
-      <c r="C134" s="22"/>
+      <c r="C134" s="15"/>
       <c r="D134" s="1"/>
       <c r="E134" s="1"/>
       <c r="F134" s="2"/>
@@ -3740,10 +3530,10 @@
       <c r="R134" s="3"/>
       <c r="S134" s="6"/>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A135" s="4"/>
       <c r="B135" s="1"/>
-      <c r="C135" s="22"/>
+      <c r="C135" s="15"/>
       <c r="D135" s="1"/>
       <c r="E135" s="1"/>
       <c r="F135" s="2"/>
@@ -3761,10 +3551,10 @@
       <c r="R135" s="3"/>
       <c r="S135" s="6"/>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A136" s="4"/>
       <c r="B136" s="1"/>
-      <c r="C136" s="22"/>
+      <c r="C136" s="15"/>
       <c r="D136" s="1"/>
       <c r="E136" s="1"/>
       <c r="F136" s="2"/>
@@ -3782,10 +3572,10 @@
       <c r="R136" s="3"/>
       <c r="S136" s="6"/>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A137" s="4"/>
       <c r="B137" s="1"/>
-      <c r="C137" s="22"/>
+      <c r="C137" s="15"/>
       <c r="D137" s="1"/>
       <c r="E137" s="1"/>
       <c r="F137" s="2"/>
@@ -3803,10 +3593,10 @@
       <c r="R137" s="3"/>
       <c r="S137" s="6"/>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A138" s="4"/>
       <c r="B138" s="1"/>
-      <c r="C138" s="22"/>
+      <c r="C138" s="15"/>
       <c r="D138" s="1"/>
       <c r="E138" s="1"/>
       <c r="F138" s="2"/>
@@ -3824,10 +3614,10 @@
       <c r="R138" s="3"/>
       <c r="S138" s="6"/>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A139" s="4"/>
       <c r="B139" s="1"/>
-      <c r="C139" s="22"/>
+      <c r="C139" s="15"/>
       <c r="D139" s="1"/>
       <c r="E139" s="1"/>
       <c r="F139" s="2"/>
@@ -3845,10 +3635,10 @@
       <c r="R139" s="3"/>
       <c r="S139" s="6"/>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A140" s="4"/>
       <c r="B140" s="1"/>
-      <c r="C140" s="22"/>
+      <c r="C140" s="15"/>
       <c r="D140" s="1"/>
       <c r="E140" s="1"/>
       <c r="F140" s="2"/>
@@ -3866,10 +3656,10 @@
       <c r="R140" s="3"/>
       <c r="S140" s="6"/>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A141" s="4"/>
       <c r="B141" s="1"/>
-      <c r="C141" s="22"/>
+      <c r="C141" s="15"/>
       <c r="D141" s="1"/>
       <c r="E141" s="1"/>
       <c r="F141" s="2"/>
@@ -3887,10 +3677,10 @@
       <c r="R141" s="3"/>
       <c r="S141" s="6"/>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A142" s="4"/>
       <c r="B142" s="1"/>
-      <c r="C142" s="22"/>
+      <c r="C142" s="15"/>
       <c r="D142" s="1"/>
       <c r="E142" s="1"/>
       <c r="F142" s="2"/>
@@ -3908,10 +3698,10 @@
       <c r="R142" s="3"/>
       <c r="S142" s="6"/>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A143" s="4"/>
       <c r="B143" s="1"/>
-      <c r="C143" s="22"/>
+      <c r="C143" s="15"/>
       <c r="D143" s="1"/>
       <c r="E143" s="1"/>
       <c r="F143" s="2"/>
@@ -3929,10 +3719,10 @@
       <c r="R143" s="3"/>
       <c r="S143" s="6"/>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A144" s="4"/>
       <c r="B144" s="1"/>
-      <c r="C144" s="22"/>
+      <c r="C144" s="15"/>
       <c r="D144" s="1"/>
       <c r="E144" s="1"/>
       <c r="F144" s="2"/>
@@ -3950,10 +3740,10 @@
       <c r="R144" s="3"/>
       <c r="S144" s="6"/>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A145" s="4"/>
       <c r="B145" s="1"/>
-      <c r="C145" s="22"/>
+      <c r="C145" s="15"/>
       <c r="D145" s="1"/>
       <c r="E145" s="1"/>
       <c r="F145" s="2"/>
@@ -3971,10 +3761,10 @@
       <c r="R145" s="3"/>
       <c r="S145" s="6"/>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A146" s="4"/>
       <c r="B146" s="1"/>
-      <c r="C146" s="22"/>
+      <c r="C146" s="15"/>
       <c r="D146" s="1"/>
       <c r="E146" s="1"/>
       <c r="F146" s="2"/>
@@ -3992,10 +3782,10 @@
       <c r="R146" s="3"/>
       <c r="S146" s="6"/>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A147" s="4"/>
       <c r="B147" s="1"/>
-      <c r="C147" s="22"/>
+      <c r="C147" s="15"/>
       <c r="D147" s="1"/>
       <c r="E147" s="1"/>
       <c r="F147" s="2"/>
@@ -4013,10 +3803,10 @@
       <c r="R147" s="3"/>
       <c r="S147" s="6"/>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A148" s="4"/>
       <c r="B148" s="1"/>
-      <c r="C148" s="22"/>
+      <c r="C148" s="15"/>
       <c r="D148" s="1"/>
       <c r="E148" s="1"/>
       <c r="F148" s="2"/>
@@ -4034,10 +3824,10 @@
       <c r="R148" s="3"/>
       <c r="S148" s="6"/>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A149" s="4"/>
       <c r="B149" s="1"/>
-      <c r="C149" s="22"/>
+      <c r="C149" s="15"/>
       <c r="D149" s="1"/>
       <c r="E149" s="1"/>
       <c r="F149" s="2"/>
@@ -4055,10 +3845,10 @@
       <c r="R149" s="3"/>
       <c r="S149" s="6"/>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A150" s="4"/>
       <c r="B150" s="1"/>
-      <c r="C150" s="22"/>
+      <c r="C150" s="15"/>
       <c r="D150" s="1"/>
       <c r="E150" s="1"/>
       <c r="F150" s="2"/>
@@ -4076,10 +3866,10 @@
       <c r="R150" s="3"/>
       <c r="S150" s="6"/>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A151" s="4"/>
       <c r="B151" s="1"/>
-      <c r="C151" s="22"/>
+      <c r="C151" s="15"/>
       <c r="D151" s="1"/>
       <c r="E151" s="1"/>
       <c r="F151" s="2"/>
@@ -4097,10 +3887,10 @@
       <c r="R151" s="3"/>
       <c r="S151" s="6"/>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A152" s="4"/>
       <c r="B152" s="1"/>
-      <c r="C152" s="22"/>
+      <c r="C152" s="15"/>
       <c r="D152" s="1"/>
       <c r="E152" s="1"/>
       <c r="F152" s="2"/>
@@ -4118,10 +3908,10 @@
       <c r="R152" s="3"/>
       <c r="S152" s="6"/>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A153" s="4"/>
       <c r="B153" s="1"/>
-      <c r="C153" s="22"/>
+      <c r="C153" s="15"/>
       <c r="D153" s="1"/>
       <c r="E153" s="1"/>
       <c r="F153" s="2"/>
@@ -4139,10 +3929,10 @@
       <c r="R153" s="3"/>
       <c r="S153" s="6"/>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A154" s="4"/>
       <c r="B154" s="1"/>
-      <c r="C154" s="22"/>
+      <c r="C154" s="15"/>
       <c r="D154" s="1"/>
       <c r="E154" s="1"/>
       <c r="F154" s="2"/>
@@ -4160,10 +3950,10 @@
       <c r="R154" s="3"/>
       <c r="S154" s="6"/>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A155" s="4"/>
       <c r="B155" s="1"/>
-      <c r="C155" s="22"/>
+      <c r="C155" s="15"/>
       <c r="D155" s="1"/>
       <c r="E155" s="1"/>
       <c r="F155" s="2"/>
@@ -4181,10 +3971,10 @@
       <c r="R155" s="3"/>
       <c r="S155" s="6"/>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A156" s="4"/>
       <c r="B156" s="1"/>
-      <c r="C156" s="22"/>
+      <c r="C156" s="15"/>
       <c r="D156" s="1"/>
       <c r="E156" s="1"/>
       <c r="F156" s="2"/>
@@ -4202,10 +3992,10 @@
       <c r="R156" s="3"/>
       <c r="S156" s="6"/>
     </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A157" s="4"/>
       <c r="B157" s="1"/>
-      <c r="C157" s="22"/>
+      <c r="C157" s="15"/>
       <c r="D157" s="1"/>
       <c r="E157" s="1"/>
       <c r="F157" s="2"/>
@@ -4223,10 +4013,10 @@
       <c r="R157" s="3"/>
       <c r="S157" s="6"/>
     </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A158" s="4"/>
       <c r="B158" s="1"/>
-      <c r="C158" s="22"/>
+      <c r="C158" s="15"/>
       <c r="D158" s="1"/>
       <c r="E158" s="1"/>
       <c r="F158" s="2"/>
@@ -4244,10 +4034,10 @@
       <c r="R158" s="3"/>
       <c r="S158" s="6"/>
     </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A159" s="4"/>
       <c r="B159" s="1"/>
-      <c r="C159" s="22"/>
+      <c r="C159" s="15"/>
       <c r="D159" s="1"/>
       <c r="E159" s="1"/>
       <c r="F159" s="2"/>
@@ -4265,10 +4055,10 @@
       <c r="R159" s="3"/>
       <c r="S159" s="6"/>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A160" s="4"/>
       <c r="B160" s="1"/>
-      <c r="C160" s="22"/>
+      <c r="C160" s="15"/>
       <c r="D160" s="1"/>
       <c r="E160" s="1"/>
       <c r="F160" s="2"/>
@@ -4286,10 +4076,10 @@
       <c r="R160" s="3"/>
       <c r="S160" s="6"/>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A161" s="4"/>
       <c r="B161" s="1"/>
-      <c r="C161" s="22"/>
+      <c r="C161" s="15"/>
       <c r="D161" s="1"/>
       <c r="E161" s="1"/>
       <c r="F161" s="2"/>
@@ -4307,10 +4097,10 @@
       <c r="R161" s="3"/>
       <c r="S161" s="6"/>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A162" s="4"/>
       <c r="B162" s="1"/>
-      <c r="C162" s="22"/>
+      <c r="C162" s="15"/>
       <c r="D162" s="1"/>
       <c r="E162" s="1"/>
       <c r="F162" s="2"/>
@@ -4328,10 +4118,10 @@
       <c r="R162" s="3"/>
       <c r="S162" s="6"/>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A163" s="4"/>
       <c r="B163" s="1"/>
-      <c r="C163" s="22"/>
+      <c r="C163" s="15"/>
       <c r="D163" s="1"/>
       <c r="E163" s="1"/>
       <c r="F163" s="2"/>
@@ -4349,10 +4139,10 @@
       <c r="R163" s="3"/>
       <c r="S163" s="6"/>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A164" s="4"/>
       <c r="B164" s="1"/>
-      <c r="C164" s="22"/>
+      <c r="C164" s="15"/>
       <c r="D164" s="1"/>
       <c r="E164" s="1"/>
       <c r="F164" s="2"/>
@@ -4370,10 +4160,10 @@
       <c r="R164" s="3"/>
       <c r="S164" s="6"/>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A165" s="4"/>
       <c r="B165" s="1"/>
-      <c r="C165" s="22"/>
+      <c r="C165" s="15"/>
       <c r="D165" s="1"/>
       <c r="E165" s="1"/>
       <c r="F165" s="2"/>
@@ -4391,10 +4181,10 @@
       <c r="R165" s="3"/>
       <c r="S165" s="6"/>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A166" s="4"/>
       <c r="B166" s="1"/>
-      <c r="C166" s="22"/>
+      <c r="C166" s="15"/>
       <c r="D166" s="1"/>
       <c r="E166" s="1"/>
       <c r="F166" s="2"/>
@@ -4412,10 +4202,10 @@
       <c r="R166" s="3"/>
       <c r="S166" s="6"/>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A167" s="4"/>
       <c r="B167" s="1"/>
-      <c r="C167" s="22"/>
+      <c r="C167" s="15"/>
       <c r="D167" s="1"/>
       <c r="E167" s="1"/>
       <c r="F167" s="2"/>
@@ -4433,10 +4223,10 @@
       <c r="R167" s="3"/>
       <c r="S167" s="6"/>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A168" s="4"/>
       <c r="B168" s="1"/>
-      <c r="C168" s="22"/>
+      <c r="C168" s="15"/>
       <c r="D168" s="1"/>
       <c r="E168" s="1"/>
       <c r="F168" s="2"/>
@@ -4454,10 +4244,10 @@
       <c r="R168" s="3"/>
       <c r="S168" s="6"/>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A169" s="4"/>
       <c r="B169" s="1"/>
-      <c r="C169" s="22"/>
+      <c r="C169" s="15"/>
       <c r="D169" s="1"/>
       <c r="E169" s="1"/>
       <c r="F169" s="2"/>
@@ -4475,10 +4265,10 @@
       <c r="R169" s="3"/>
       <c r="S169" s="6"/>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A170" s="4"/>
       <c r="B170" s="1"/>
-      <c r="C170" s="22"/>
+      <c r="C170" s="15"/>
       <c r="D170" s="1"/>
       <c r="E170" s="1"/>
       <c r="F170" s="2"/>
@@ -4496,10 +4286,10 @@
       <c r="R170" s="3"/>
       <c r="S170" s="6"/>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A171" s="4"/>
       <c r="B171" s="1"/>
-      <c r="C171" s="22"/>
+      <c r="C171" s="15"/>
       <c r="D171" s="1"/>
       <c r="E171" s="1"/>
       <c r="F171" s="2"/>
@@ -4517,10 +4307,10 @@
       <c r="R171" s="3"/>
       <c r="S171" s="6"/>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A172" s="4"/>
       <c r="B172" s="1"/>
-      <c r="C172" s="22"/>
+      <c r="C172" s="15"/>
       <c r="D172" s="1"/>
       <c r="E172" s="1"/>
       <c r="F172" s="2"/>
@@ -4538,10 +4328,10 @@
       <c r="R172" s="3"/>
       <c r="S172" s="6"/>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A173" s="4"/>
       <c r="B173" s="1"/>
-      <c r="C173" s="22"/>
+      <c r="C173" s="15"/>
       <c r="D173" s="1"/>
       <c r="E173" s="1"/>
       <c r="F173" s="2"/>
@@ -4559,10 +4349,10 @@
       <c r="R173" s="3"/>
       <c r="S173" s="6"/>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A174" s="4"/>
       <c r="B174" s="1"/>
-      <c r="C174" s="22"/>
+      <c r="C174" s="15"/>
       <c r="D174" s="1"/>
       <c r="E174" s="1"/>
       <c r="F174" s="2"/>
@@ -4580,10 +4370,10 @@
       <c r="R174" s="3"/>
       <c r="S174" s="6"/>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A175" s="4"/>
       <c r="B175" s="1"/>
-      <c r="C175" s="22"/>
+      <c r="C175" s="15"/>
       <c r="D175" s="1"/>
       <c r="E175" s="1"/>
       <c r="F175" s="2"/>
@@ -4601,10 +4391,10 @@
       <c r="R175" s="3"/>
       <c r="S175" s="6"/>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A176" s="4"/>
       <c r="B176" s="1"/>
-      <c r="C176" s="22"/>
+      <c r="C176" s="15"/>
       <c r="D176" s="1"/>
       <c r="E176" s="1"/>
       <c r="F176" s="2"/>
@@ -4622,10 +4412,10 @@
       <c r="R176" s="3"/>
       <c r="S176" s="6"/>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A177" s="4"/>
       <c r="B177" s="1"/>
-      <c r="C177" s="22"/>
+      <c r="C177" s="15"/>
       <c r="D177" s="1"/>
       <c r="E177" s="1"/>
       <c r="F177" s="2"/>
@@ -4643,10 +4433,10 @@
       <c r="R177" s="3"/>
       <c r="S177" s="6"/>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A178" s="4"/>
       <c r="B178" s="1"/>
-      <c r="C178" s="22"/>
+      <c r="C178" s="15"/>
       <c r="D178" s="1"/>
       <c r="E178" s="1"/>
       <c r="F178" s="2"/>
@@ -4664,10 +4454,10 @@
       <c r="R178" s="3"/>
       <c r="S178" s="6"/>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A179" s="4"/>
       <c r="B179" s="1"/>
-      <c r="C179" s="22"/>
+      <c r="C179" s="15"/>
       <c r="D179" s="1"/>
       <c r="E179" s="1"/>
       <c r="F179" s="2"/>
@@ -4685,10 +4475,10 @@
       <c r="R179" s="3"/>
       <c r="S179" s="6"/>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A180" s="4"/>
       <c r="B180" s="1"/>
-      <c r="C180" s="22"/>
+      <c r="C180" s="15"/>
       <c r="D180" s="1"/>
       <c r="E180" s="1"/>
       <c r="F180" s="2"/>
@@ -4706,10 +4496,10 @@
       <c r="R180" s="3"/>
       <c r="S180" s="6"/>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A181" s="4"/>
       <c r="B181" s="1"/>
-      <c r="C181" s="22"/>
+      <c r="C181" s="15"/>
       <c r="D181" s="1"/>
       <c r="E181" s="1"/>
       <c r="F181" s="2"/>
@@ -4727,10 +4517,10 @@
       <c r="R181" s="3"/>
       <c r="S181" s="6"/>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A182" s="4"/>
       <c r="B182" s="1"/>
-      <c r="C182" s="22"/>
+      <c r="C182" s="15"/>
       <c r="D182" s="1"/>
       <c r="E182" s="1"/>
       <c r="F182" s="2"/>
@@ -4748,10 +4538,10 @@
       <c r="R182" s="3"/>
       <c r="S182" s="6"/>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A183" s="4"/>
       <c r="B183" s="1"/>
-      <c r="C183" s="22"/>
+      <c r="C183" s="15"/>
       <c r="D183" s="1"/>
       <c r="E183" s="1"/>
       <c r="F183" s="2"/>
@@ -4769,10 +4559,10 @@
       <c r="R183" s="3"/>
       <c r="S183" s="6"/>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A184" s="4"/>
       <c r="B184" s="1"/>
-      <c r="C184" s="22"/>
+      <c r="C184" s="15"/>
       <c r="D184" s="1"/>
       <c r="E184" s="1"/>
       <c r="F184" s="2"/>
@@ -4790,10 +4580,10 @@
       <c r="R184" s="3"/>
       <c r="S184" s="6"/>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A185" s="4"/>
       <c r="B185" s="1"/>
-      <c r="C185" s="22"/>
+      <c r="C185" s="15"/>
       <c r="D185" s="1"/>
       <c r="E185" s="1"/>
       <c r="F185" s="2"/>
@@ -4811,10 +4601,10 @@
       <c r="R185" s="3"/>
       <c r="S185" s="6"/>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A186" s="4"/>
       <c r="B186" s="1"/>
-      <c r="C186" s="22"/>
+      <c r="C186" s="15"/>
       <c r="D186" s="1"/>
       <c r="E186" s="1"/>
       <c r="F186" s="2"/>
@@ -4832,10 +4622,10 @@
       <c r="R186" s="3"/>
       <c r="S186" s="6"/>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A187" s="4"/>
       <c r="B187" s="1"/>
-      <c r="C187" s="22"/>
+      <c r="C187" s="15"/>
       <c r="D187" s="1"/>
       <c r="E187" s="1"/>
       <c r="F187" s="2"/>
@@ -4853,10 +4643,10 @@
       <c r="R187" s="3"/>
       <c r="S187" s="6"/>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A188" s="4"/>
       <c r="B188" s="1"/>
-      <c r="C188" s="22"/>
+      <c r="C188" s="15"/>
       <c r="D188" s="1"/>
       <c r="E188" s="1"/>
       <c r="F188" s="2"/>
@@ -4874,10 +4664,10 @@
       <c r="R188" s="3"/>
       <c r="S188" s="6"/>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A189" s="4"/>
       <c r="B189" s="1"/>
-      <c r="C189" s="22"/>
+      <c r="C189" s="15"/>
       <c r="D189" s="1"/>
       <c r="E189" s="1"/>
       <c r="F189" s="2"/>
@@ -4895,10 +4685,10 @@
       <c r="R189" s="3"/>
       <c r="S189" s="6"/>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A190" s="4"/>
       <c r="B190" s="1"/>
-      <c r="C190" s="22"/>
+      <c r="C190" s="15"/>
       <c r="D190" s="1"/>
       <c r="E190" s="1"/>
       <c r="F190" s="2"/>
@@ -4916,10 +4706,10 @@
       <c r="R190" s="3"/>
       <c r="S190" s="6"/>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A191" s="4"/>
       <c r="B191" s="1"/>
-      <c r="C191" s="22"/>
+      <c r="C191" s="15"/>
       <c r="D191" s="1"/>
       <c r="E191" s="1"/>
       <c r="F191" s="2"/>
@@ -4937,10 +4727,10 @@
       <c r="R191" s="3"/>
       <c r="S191" s="6"/>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A192" s="4"/>
       <c r="B192" s="1"/>
-      <c r="C192" s="22"/>
+      <c r="C192" s="15"/>
       <c r="D192" s="1"/>
       <c r="E192" s="1"/>
       <c r="F192" s="2"/>
@@ -4958,10 +4748,10 @@
       <c r="R192" s="3"/>
       <c r="S192" s="6"/>
     </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A193" s="4"/>
       <c r="B193" s="1"/>
-      <c r="C193" s="22"/>
+      <c r="C193" s="15"/>
       <c r="D193" s="1"/>
       <c r="E193" s="1"/>
       <c r="F193" s="2"/>
@@ -4979,10 +4769,10 @@
       <c r="R193" s="3"/>
       <c r="S193" s="6"/>
     </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A194" s="4"/>
       <c r="B194" s="1"/>
-      <c r="C194" s="22"/>
+      <c r="C194" s="15"/>
       <c r="D194" s="1"/>
       <c r="E194" s="1"/>
       <c r="F194" s="2"/>
@@ -5000,10 +4790,10 @@
       <c r="R194" s="3"/>
       <c r="S194" s="6"/>
     </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A195" s="4"/>
       <c r="B195" s="1"/>
-      <c r="C195" s="22"/>
+      <c r="C195" s="15"/>
       <c r="D195" s="1"/>
       <c r="E195" s="1"/>
       <c r="F195" s="2"/>
@@ -5021,10 +4811,10 @@
       <c r="R195" s="3"/>
       <c r="S195" s="6"/>
     </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A196" s="4"/>
       <c r="B196" s="1"/>
-      <c r="C196" s="22"/>
+      <c r="C196" s="15"/>
       <c r="D196" s="1"/>
       <c r="E196" s="1"/>
       <c r="F196" s="2"/>
@@ -5042,10 +4832,10 @@
       <c r="R196" s="3"/>
       <c r="S196" s="6"/>
     </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A197" s="4"/>
       <c r="B197" s="1"/>
-      <c r="C197" s="22"/>
+      <c r="C197" s="15"/>
       <c r="D197" s="1"/>
       <c r="E197" s="1"/>
       <c r="F197" s="2"/>
@@ -5063,10 +4853,10 @@
       <c r="R197" s="3"/>
       <c r="S197" s="6"/>
     </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A198" s="4"/>
       <c r="B198" s="1"/>
-      <c r="C198" s="22"/>
+      <c r="C198" s="15"/>
       <c r="D198" s="1"/>
       <c r="E198" s="1"/>
       <c r="F198" s="2"/>
@@ -5084,10 +4874,10 @@
       <c r="R198" s="3"/>
       <c r="S198" s="6"/>
     </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A199" s="4"/>
       <c r="B199" s="1"/>
-      <c r="C199" s="22"/>
+      <c r="C199" s="15"/>
       <c r="D199" s="1"/>
       <c r="E199" s="1"/>
       <c r="F199" s="2"/>
@@ -5105,10 +4895,10 @@
       <c r="R199" s="3"/>
       <c r="S199" s="6"/>
     </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A200" s="4"/>
       <c r="B200" s="1"/>
-      <c r="C200" s="22"/>
+      <c r="C200" s="15"/>
       <c r="D200" s="1"/>
       <c r="E200" s="1"/>
       <c r="F200" s="2"/>
@@ -5126,10 +4916,10 @@
       <c r="R200" s="3"/>
       <c r="S200" s="6"/>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A201" s="4"/>
       <c r="B201" s="1"/>
-      <c r="C201" s="22"/>
+      <c r="C201" s="15"/>
       <c r="D201" s="1"/>
       <c r="E201" s="1"/>
       <c r="F201" s="2"/>
@@ -5147,10 +4937,10 @@
       <c r="R201" s="3"/>
       <c r="S201" s="6"/>
     </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A202" s="4"/>
       <c r="B202" s="1"/>
-      <c r="C202" s="22"/>
+      <c r="C202" s="15"/>
       <c r="D202" s="1"/>
       <c r="E202" s="1"/>
       <c r="F202" s="2"/>
@@ -5168,10 +4958,10 @@
       <c r="R202" s="3"/>
       <c r="S202" s="6"/>
     </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A203" s="4"/>
       <c r="B203" s="1"/>
-      <c r="C203" s="22"/>
+      <c r="C203" s="15"/>
       <c r="D203" s="1"/>
       <c r="E203" s="1"/>
       <c r="F203" s="2"/>
@@ -5189,10 +4979,10 @@
       <c r="R203" s="3"/>
       <c r="S203" s="6"/>
     </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A204" s="4"/>
       <c r="B204" s="1"/>
-      <c r="C204" s="22"/>
+      <c r="C204" s="15"/>
       <c r="D204" s="1"/>
       <c r="E204" s="1"/>
       <c r="F204" s="2"/>
@@ -5210,10 +5000,10 @@
       <c r="R204" s="3"/>
       <c r="S204" s="6"/>
     </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A205" s="4"/>
       <c r="B205" s="1"/>
-      <c r="C205" s="22"/>
+      <c r="C205" s="15"/>
       <c r="D205" s="1"/>
       <c r="E205" s="1"/>
       <c r="F205" s="2"/>
@@ -5231,10 +5021,10 @@
       <c r="R205" s="3"/>
       <c r="S205" s="6"/>
     </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A206" s="4"/>
       <c r="B206" s="1"/>
-      <c r="C206" s="22"/>
+      <c r="C206" s="15"/>
       <c r="D206" s="1"/>
       <c r="E206" s="1"/>
       <c r="F206" s="2"/>
@@ -5252,10 +5042,10 @@
       <c r="R206" s="3"/>
       <c r="S206" s="6"/>
     </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A207" s="4"/>
       <c r="B207" s="1"/>
-      <c r="C207" s="22"/>
+      <c r="C207" s="15"/>
       <c r="D207" s="1"/>
       <c r="E207" s="1"/>
       <c r="F207" s="2"/>
@@ -5273,10 +5063,10 @@
       <c r="R207" s="3"/>
       <c r="S207" s="6"/>
     </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A208" s="4"/>
       <c r="B208" s="1"/>
-      <c r="C208" s="22"/>
+      <c r="C208" s="15"/>
       <c r="D208" s="1"/>
       <c r="E208" s="1"/>
       <c r="F208" s="2"/>
@@ -5294,10 +5084,10 @@
       <c r="R208" s="3"/>
       <c r="S208" s="6"/>
     </row>
-    <row r="209" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A209" s="4"/>
       <c r="B209" s="1"/>
-      <c r="C209" s="22"/>
+      <c r="C209" s="15"/>
       <c r="D209" s="1"/>
       <c r="E209" s="1"/>
       <c r="F209" s="2"/>
@@ -5315,10 +5105,10 @@
       <c r="R209" s="3"/>
       <c r="S209" s="6"/>
     </row>
-    <row r="210" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A210" s="4"/>
       <c r="B210" s="1"/>
-      <c r="C210" s="22"/>
+      <c r="C210" s="15"/>
       <c r="D210" s="1"/>
       <c r="E210" s="1"/>
       <c r="F210" s="2"/>
@@ -5336,10 +5126,10 @@
       <c r="R210" s="3"/>
       <c r="S210" s="6"/>
     </row>
-    <row r="211" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A211" s="4"/>
       <c r="B211" s="1"/>
-      <c r="C211" s="22"/>
+      <c r="C211" s="15"/>
       <c r="D211" s="1"/>
       <c r="E211" s="1"/>
       <c r="F211" s="2"/>
@@ -5357,10 +5147,10 @@
       <c r="R211" s="3"/>
       <c r="S211" s="6"/>
     </row>
-    <row r="212" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A212" s="4"/>
       <c r="B212" s="1"/>
-      <c r="C212" s="22"/>
+      <c r="C212" s="15"/>
       <c r="D212" s="1"/>
       <c r="E212" s="1"/>
       <c r="F212" s="2"/>
@@ -5378,10 +5168,10 @@
       <c r="R212" s="3"/>
       <c r="S212" s="6"/>
     </row>
-    <row r="213" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A213" s="4"/>
       <c r="B213" s="1"/>
-      <c r="C213" s="22"/>
+      <c r="C213" s="15"/>
       <c r="D213" s="1"/>
       <c r="E213" s="1"/>
       <c r="F213" s="2"/>
@@ -5399,10 +5189,10 @@
       <c r="R213" s="3"/>
       <c r="S213" s="6"/>
     </row>
-    <row r="214" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A214" s="4"/>
       <c r="B214" s="1"/>
-      <c r="C214" s="22"/>
+      <c r="C214" s="15"/>
       <c r="D214" s="1"/>
       <c r="E214" s="1"/>
       <c r="F214" s="2"/>
@@ -5420,10 +5210,10 @@
       <c r="R214" s="3"/>
       <c r="S214" s="6"/>
     </row>
-    <row r="215" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A215" s="4"/>
       <c r="B215" s="1"/>
-      <c r="C215" s="22"/>
+      <c r="C215" s="15"/>
       <c r="D215" s="1"/>
       <c r="E215" s="1"/>
       <c r="F215" s="2"/>
@@ -5441,10 +5231,10 @@
       <c r="R215" s="3"/>
       <c r="S215" s="6"/>
     </row>
-    <row r="216" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A216" s="4"/>
       <c r="B216" s="1"/>
-      <c r="C216" s="22"/>
+      <c r="C216" s="15"/>
       <c r="D216" s="1"/>
       <c r="E216" s="1"/>
       <c r="F216" s="2"/>
@@ -5462,10 +5252,10 @@
       <c r="R216" s="3"/>
       <c r="S216" s="6"/>
     </row>
-    <row r="217" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A217" s="4"/>
       <c r="B217" s="1"/>
-      <c r="C217" s="22"/>
+      <c r="C217" s="15"/>
       <c r="D217" s="1"/>
       <c r="E217" s="1"/>
       <c r="F217" s="2"/>
@@ -5483,10 +5273,10 @@
       <c r="R217" s="3"/>
       <c r="S217" s="6"/>
     </row>
-    <row r="218" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A218" s="4"/>
       <c r="B218" s="1"/>
-      <c r="C218" s="22"/>
+      <c r="C218" s="15"/>
       <c r="D218" s="1"/>
       <c r="E218" s="1"/>
       <c r="F218" s="2"/>
@@ -5504,10 +5294,10 @@
       <c r="R218" s="3"/>
       <c r="S218" s="6"/>
     </row>
-    <row r="219" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A219" s="4"/>
       <c r="B219" s="1"/>
-      <c r="C219" s="22"/>
+      <c r="C219" s="15"/>
       <c r="D219" s="1"/>
       <c r="E219" s="1"/>
       <c r="F219" s="2"/>
@@ -5525,10 +5315,10 @@
       <c r="R219" s="3"/>
       <c r="S219" s="6"/>
     </row>
-    <row r="220" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A220" s="4"/>
       <c r="B220" s="1"/>
-      <c r="C220" s="22"/>
+      <c r="C220" s="15"/>
       <c r="D220" s="1"/>
       <c r="E220" s="1"/>
       <c r="F220" s="2"/>
@@ -5546,10 +5336,10 @@
       <c r="R220" s="3"/>
       <c r="S220" s="6"/>
     </row>
-    <row r="221" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A221" s="4"/>
       <c r="B221" s="1"/>
-      <c r="C221" s="22"/>
+      <c r="C221" s="15"/>
       <c r="D221" s="1"/>
       <c r="E221" s="1"/>
       <c r="F221" s="2"/>
@@ -5567,10 +5357,10 @@
       <c r="R221" s="3"/>
       <c r="S221" s="6"/>
     </row>
-    <row r="222" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A222" s="4"/>
       <c r="B222" s="1"/>
-      <c r="C222" s="22"/>
+      <c r="C222" s="15"/>
       <c r="D222" s="1"/>
       <c r="E222" s="1"/>
       <c r="F222" s="2"/>
@@ -5588,10 +5378,10 @@
       <c r="R222" s="3"/>
       <c r="S222" s="6"/>
     </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A223" s="4"/>
       <c r="B223" s="1"/>
-      <c r="C223" s="22"/>
+      <c r="C223" s="15"/>
       <c r="D223" s="1"/>
       <c r="E223" s="1"/>
       <c r="F223" s="2"/>
@@ -5609,10 +5399,10 @@
       <c r="R223" s="3"/>
       <c r="S223" s="6"/>
     </row>
-    <row r="224" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A224" s="4"/>
       <c r="B224" s="1"/>
-      <c r="C224" s="22"/>
+      <c r="C224" s="15"/>
       <c r="D224" s="1"/>
       <c r="E224" s="1"/>
       <c r="F224" s="2"/>
@@ -5630,10 +5420,10 @@
       <c r="R224" s="3"/>
       <c r="S224" s="6"/>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A225" s="4"/>
       <c r="B225" s="1"/>
-      <c r="C225" s="22"/>
+      <c r="C225" s="15"/>
       <c r="D225" s="1"/>
       <c r="E225" s="1"/>
       <c r="F225" s="2"/>
@@ -5651,10 +5441,10 @@
       <c r="R225" s="3"/>
       <c r="S225" s="6"/>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A226" s="4"/>
       <c r="B226" s="1"/>
-      <c r="C226" s="22"/>
+      <c r="C226" s="15"/>
       <c r="D226" s="1"/>
       <c r="E226" s="1"/>
       <c r="F226" s="2"/>
@@ -5672,10 +5462,10 @@
       <c r="R226" s="3"/>
       <c r="S226" s="6"/>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A227" s="4"/>
       <c r="B227" s="1"/>
-      <c r="C227" s="22"/>
+      <c r="C227" s="15"/>
       <c r="D227" s="1"/>
       <c r="E227" s="1"/>
       <c r="F227" s="2"/>
@@ -5693,10 +5483,10 @@
       <c r="R227" s="3"/>
       <c r="S227" s="6"/>
     </row>
-    <row r="228" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A228" s="4"/>
       <c r="B228" s="1"/>
-      <c r="C228" s="22"/>
+      <c r="C228" s="15"/>
       <c r="D228" s="1"/>
       <c r="E228" s="1"/>
       <c r="F228" s="2"/>
@@ -5714,10 +5504,10 @@
       <c r="R228" s="3"/>
       <c r="S228" s="6"/>
     </row>
-    <row r="229" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A229" s="4"/>
       <c r="B229" s="1"/>
-      <c r="C229" s="22"/>
+      <c r="C229" s="15"/>
       <c r="D229" s="1"/>
       <c r="E229" s="1"/>
       <c r="F229" s="2"/>
@@ -5735,10 +5525,10 @@
       <c r="R229" s="3"/>
       <c r="S229" s="6"/>
     </row>
-    <row r="230" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A230" s="4"/>
       <c r="B230" s="1"/>
-      <c r="C230" s="22"/>
+      <c r="C230" s="15"/>
       <c r="D230" s="1"/>
       <c r="E230" s="1"/>
       <c r="F230" s="2"/>
@@ -5756,10 +5546,10 @@
       <c r="R230" s="3"/>
       <c r="S230" s="6"/>
     </row>
-    <row r="231" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A231" s="4"/>
       <c r="B231" s="1"/>
-      <c r="C231" s="22"/>
+      <c r="C231" s="15"/>
       <c r="D231" s="1"/>
       <c r="E231" s="1"/>
       <c r="F231" s="2"/>
@@ -5777,10 +5567,10 @@
       <c r="R231" s="3"/>
       <c r="S231" s="6"/>
     </row>
-    <row r="232" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A232" s="4"/>
       <c r="B232" s="1"/>
-      <c r="C232" s="22"/>
+      <c r="C232" s="15"/>
       <c r="D232" s="1"/>
       <c r="E232" s="1"/>
       <c r="F232" s="2"/>
@@ -5798,10 +5588,10 @@
       <c r="R232" s="3"/>
       <c r="S232" s="6"/>
     </row>
-    <row r="233" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A233" s="4"/>
       <c r="B233" s="1"/>
-      <c r="C233" s="22"/>
+      <c r="C233" s="15"/>
       <c r="D233" s="1"/>
       <c r="E233" s="1"/>
       <c r="F233" s="2"/>
@@ -5819,10 +5609,10 @@
       <c r="R233" s="3"/>
       <c r="S233" s="6"/>
     </row>
-    <row r="234" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A234" s="4"/>
       <c r="B234" s="1"/>
-      <c r="C234" s="22"/>
+      <c r="C234" s="15"/>
       <c r="D234" s="1"/>
       <c r="E234" s="1"/>
       <c r="F234" s="2"/>
@@ -5840,10 +5630,10 @@
       <c r="R234" s="3"/>
       <c r="S234" s="6"/>
     </row>
-    <row r="235" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A235" s="4"/>
       <c r="B235" s="1"/>
-      <c r="C235" s="22"/>
+      <c r="C235" s="15"/>
       <c r="D235" s="1"/>
       <c r="E235" s="1"/>
       <c r="F235" s="2"/>
@@ -5861,10 +5651,10 @@
       <c r="R235" s="3"/>
       <c r="S235" s="6"/>
     </row>
-    <row r="236" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A236" s="4"/>
       <c r="B236" s="1"/>
-      <c r="C236" s="22"/>
+      <c r="C236" s="15"/>
       <c r="D236" s="1"/>
       <c r="E236" s="1"/>
       <c r="F236" s="2"/>
@@ -5882,10 +5672,10 @@
       <c r="R236" s="3"/>
       <c r="S236" s="6"/>
     </row>
-    <row r="237" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A237" s="4"/>
       <c r="B237" s="1"/>
-      <c r="C237" s="22"/>
+      <c r="C237" s="15"/>
       <c r="D237" s="1"/>
       <c r="E237" s="1"/>
       <c r="F237" s="2"/>
@@ -5903,10 +5693,10 @@
       <c r="R237" s="3"/>
       <c r="S237" s="6"/>
     </row>
-    <row r="238" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A238" s="4"/>
       <c r="B238" s="1"/>
-      <c r="C238" s="22"/>
+      <c r="C238" s="15"/>
       <c r="D238" s="1"/>
       <c r="E238" s="1"/>
       <c r="F238" s="2"/>
@@ -5924,10 +5714,10 @@
       <c r="R238" s="3"/>
       <c r="S238" s="6"/>
     </row>
-    <row r="239" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A239" s="4"/>
       <c r="B239" s="1"/>
-      <c r="C239" s="22"/>
+      <c r="C239" s="15"/>
       <c r="D239" s="1"/>
       <c r="E239" s="1"/>
       <c r="F239" s="2"/>
@@ -5945,10 +5735,10 @@
       <c r="R239" s="3"/>
       <c r="S239" s="6"/>
     </row>
-    <row r="240" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A240" s="4"/>
       <c r="B240" s="1"/>
-      <c r="C240" s="22"/>
+      <c r="C240" s="15"/>
       <c r="D240" s="1"/>
       <c r="E240" s="1"/>
       <c r="F240" s="2"/>
@@ -5966,10 +5756,10 @@
       <c r="R240" s="3"/>
       <c r="S240" s="6"/>
     </row>
-    <row r="241" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A241" s="4"/>
       <c r="B241" s="1"/>
-      <c r="C241" s="22"/>
+      <c r="C241" s="15"/>
       <c r="D241" s="1"/>
       <c r="E241" s="1"/>
       <c r="F241" s="2"/>
@@ -5987,10 +5777,10 @@
       <c r="R241" s="3"/>
       <c r="S241" s="6"/>
     </row>
-    <row r="242" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A242" s="4"/>
       <c r="B242" s="1"/>
-      <c r="C242" s="22"/>
+      <c r="C242" s="15"/>
       <c r="D242" s="1"/>
       <c r="E242" s="1"/>
       <c r="F242" s="2"/>
@@ -6008,10 +5798,10 @@
       <c r="R242" s="3"/>
       <c r="S242" s="6"/>
     </row>
-    <row r="243" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A243" s="4"/>
       <c r="B243" s="1"/>
-      <c r="C243" s="22"/>
+      <c r="C243" s="15"/>
       <c r="D243" s="1"/>
       <c r="E243" s="1"/>
       <c r="F243" s="2"/>
@@ -6029,10 +5819,10 @@
       <c r="R243" s="3"/>
       <c r="S243" s="6"/>
     </row>
-    <row r="244" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A244" s="4"/>
       <c r="B244" s="1"/>
-      <c r="C244" s="22"/>
+      <c r="C244" s="15"/>
       <c r="D244" s="1"/>
       <c r="E244" s="1"/>
       <c r="F244" s="2"/>
@@ -6050,10 +5840,10 @@
       <c r="R244" s="3"/>
       <c r="S244" s="6"/>
     </row>
-    <row r="245" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A245" s="4"/>
       <c r="B245" s="1"/>
-      <c r="C245" s="22"/>
+      <c r="C245" s="15"/>
       <c r="D245" s="1"/>
       <c r="E245" s="1"/>
       <c r="F245" s="2"/>
@@ -6071,10 +5861,10 @@
       <c r="R245" s="3"/>
       <c r="S245" s="6"/>
     </row>
-    <row r="246" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A246" s="4"/>
       <c r="B246" s="1"/>
-      <c r="C246" s="22"/>
+      <c r="C246" s="15"/>
       <c r="D246" s="1"/>
       <c r="E246" s="1"/>
       <c r="F246" s="2"/>
@@ -6092,10 +5882,10 @@
       <c r="R246" s="3"/>
       <c r="S246" s="6"/>
     </row>
-    <row r="247" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A247" s="4"/>
       <c r="B247" s="1"/>
-      <c r="C247" s="22"/>
+      <c r="C247" s="15"/>
       <c r="D247" s="1"/>
       <c r="E247" s="1"/>
       <c r="F247" s="2"/>
@@ -6113,10 +5903,10 @@
       <c r="R247" s="3"/>
       <c r="S247" s="6"/>
     </row>
-    <row r="248" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A248" s="4"/>
       <c r="B248" s="1"/>
-      <c r="C248" s="22"/>
+      <c r="C248" s="15"/>
       <c r="D248" s="1"/>
       <c r="E248" s="1"/>
       <c r="F248" s="2"/>
@@ -6134,10 +5924,10 @@
       <c r="R248" s="3"/>
       <c r="S248" s="6"/>
     </row>
-    <row r="249" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A249" s="4"/>
       <c r="B249" s="1"/>
-      <c r="C249" s="22"/>
+      <c r="C249" s="15"/>
       <c r="D249" s="1"/>
       <c r="E249" s="1"/>
       <c r="F249" s="2"/>
@@ -6155,10 +5945,10 @@
       <c r="R249" s="3"/>
       <c r="S249" s="6"/>
     </row>
-    <row r="250" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A250" s="4"/>
       <c r="B250" s="1"/>
-      <c r="C250" s="22"/>
+      <c r="C250" s="15"/>
       <c r="D250" s="1"/>
       <c r="E250" s="1"/>
       <c r="F250" s="2"/>
@@ -6176,10 +5966,10 @@
       <c r="R250" s="3"/>
       <c r="S250" s="6"/>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A251" s="4"/>
       <c r="B251" s="1"/>
-      <c r="C251" s="22"/>
+      <c r="C251" s="15"/>
       <c r="D251" s="1"/>
       <c r="E251" s="1"/>
       <c r="F251" s="2"/>
@@ -6197,10 +5987,10 @@
       <c r="R251" s="3"/>
       <c r="S251" s="6"/>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A252" s="4"/>
       <c r="B252" s="1"/>
-      <c r="C252" s="22"/>
+      <c r="C252" s="15"/>
       <c r="D252" s="1"/>
       <c r="E252" s="1"/>
       <c r="F252" s="2"/>
@@ -6218,10 +6008,10 @@
       <c r="R252" s="3"/>
       <c r="S252" s="6"/>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A253" s="4"/>
       <c r="B253" s="1"/>
-      <c r="C253" s="22"/>
+      <c r="C253" s="15"/>
       <c r="D253" s="1"/>
       <c r="E253" s="1"/>
       <c r="F253" s="2"/>
@@ -6239,10 +6029,10 @@
       <c r="R253" s="3"/>
       <c r="S253" s="6"/>
     </row>
-    <row r="254" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A254" s="4"/>
       <c r="B254" s="1"/>
-      <c r="C254" s="22"/>
+      <c r="C254" s="15"/>
       <c r="D254" s="1"/>
       <c r="E254" s="1"/>
       <c r="F254" s="2"/>
@@ -6260,10 +6050,10 @@
       <c r="R254" s="3"/>
       <c r="S254" s="6"/>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A255" s="4"/>
       <c r="B255" s="1"/>
-      <c r="C255" s="22"/>
+      <c r="C255" s="15"/>
       <c r="D255" s="1"/>
       <c r="E255" s="1"/>
       <c r="F255" s="2"/>
@@ -6281,10 +6071,10 @@
       <c r="R255" s="3"/>
       <c r="S255" s="6"/>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A256" s="4"/>
       <c r="B256" s="1"/>
-      <c r="C256" s="22"/>
+      <c r="C256" s="15"/>
       <c r="D256" s="1"/>
       <c r="E256" s="1"/>
       <c r="F256" s="2"/>
@@ -6302,10 +6092,10 @@
       <c r="R256" s="3"/>
       <c r="S256" s="6"/>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A257" s="4"/>
       <c r="B257" s="1"/>
-      <c r="C257" s="22"/>
+      <c r="C257" s="15"/>
       <c r="D257" s="1"/>
       <c r="E257" s="1"/>
       <c r="F257" s="2"/>
@@ -6323,10 +6113,10 @@
       <c r="R257" s="3"/>
       <c r="S257" s="6"/>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A258" s="4"/>
       <c r="B258" s="1"/>
-      <c r="C258" s="22"/>
+      <c r="C258" s="15"/>
       <c r="D258" s="1"/>
       <c r="E258" s="1"/>
       <c r="F258" s="2"/>
@@ -6344,10 +6134,10 @@
       <c r="R258" s="3"/>
       <c r="S258" s="6"/>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A259" s="4"/>
       <c r="B259" s="1"/>
-      <c r="C259" s="22"/>
+      <c r="C259" s="15"/>
       <c r="D259" s="1"/>
       <c r="E259" s="1"/>
       <c r="F259" s="2"/>
@@ -6365,10 +6155,10 @@
       <c r="R259" s="3"/>
       <c r="S259" s="6"/>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A260" s="4"/>
       <c r="B260" s="1"/>
-      <c r="C260" s="22"/>
+      <c r="C260" s="15"/>
       <c r="D260" s="1"/>
       <c r="E260" s="1"/>
       <c r="F260" s="2"/>
@@ -6386,10 +6176,10 @@
       <c r="R260" s="3"/>
       <c r="S260" s="6"/>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A261" s="4"/>
       <c r="B261" s="1"/>
-      <c r="C261" s="22"/>
+      <c r="C261" s="15"/>
       <c r="D261" s="1"/>
       <c r="E261" s="1"/>
       <c r="F261" s="2"/>
@@ -6407,10 +6197,10 @@
       <c r="R261" s="3"/>
       <c r="S261" s="6"/>
     </row>
-    <row r="262" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A262" s="4"/>
       <c r="B262" s="1"/>
-      <c r="C262" s="22"/>
+      <c r="C262" s="15"/>
       <c r="D262" s="1"/>
       <c r="E262" s="1"/>
       <c r="F262" s="2"/>
@@ -6428,10 +6218,10 @@
       <c r="R262" s="3"/>
       <c r="S262" s="6"/>
     </row>
-    <row r="263" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A263" s="4"/>
       <c r="B263" s="1"/>
-      <c r="C263" s="22"/>
+      <c r="C263" s="15"/>
       <c r="D263" s="1"/>
       <c r="E263" s="1"/>
       <c r="F263" s="2"/>
@@ -6449,10 +6239,10 @@
       <c r="R263" s="3"/>
       <c r="S263" s="6"/>
     </row>
-    <row r="264" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A264" s="4"/>
       <c r="B264" s="1"/>
-      <c r="C264" s="22"/>
+      <c r="C264" s="15"/>
       <c r="D264" s="1"/>
       <c r="E264" s="1"/>
       <c r="F264" s="2"/>
@@ -6470,10 +6260,10 @@
       <c r="R264" s="3"/>
       <c r="S264" s="6"/>
     </row>
-    <row r="265" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A265" s="4"/>
       <c r="B265" s="1"/>
-      <c r="C265" s="22"/>
+      <c r="C265" s="15"/>
       <c r="D265" s="1"/>
       <c r="E265" s="1"/>
       <c r="F265" s="2"/>
@@ -6491,10 +6281,10 @@
       <c r="R265" s="3"/>
       <c r="S265" s="6"/>
     </row>
-    <row r="266" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A266" s="4"/>
       <c r="B266" s="1"/>
-      <c r="C266" s="22"/>
+      <c r="C266" s="15"/>
       <c r="D266" s="1"/>
       <c r="E266" s="1"/>
       <c r="F266" s="2"/>
@@ -6512,10 +6302,10 @@
       <c r="R266" s="3"/>
       <c r="S266" s="6"/>
     </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A267" s="4"/>
       <c r="B267" s="1"/>
-      <c r="C267" s="22"/>
+      <c r="C267" s="15"/>
       <c r="D267" s="1"/>
       <c r="E267" s="1"/>
       <c r="F267" s="2"/>
@@ -6533,10 +6323,10 @@
       <c r="R267" s="3"/>
       <c r="S267" s="6"/>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A268" s="4"/>
       <c r="B268" s="1"/>
-      <c r="C268" s="22"/>
+      <c r="C268" s="15"/>
       <c r="D268" s="1"/>
       <c r="E268" s="1"/>
       <c r="F268" s="2"/>
@@ -6554,10 +6344,10 @@
       <c r="R268" s="3"/>
       <c r="S268" s="6"/>
     </row>
-    <row r="269" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A269" s="4"/>
       <c r="B269" s="1"/>
-      <c r="C269" s="22"/>
+      <c r="C269" s="15"/>
       <c r="D269" s="1"/>
       <c r="E269" s="1"/>
       <c r="F269" s="2"/>
@@ -6575,10 +6365,10 @@
       <c r="R269" s="3"/>
       <c r="S269" s="6"/>
     </row>
-    <row r="270" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A270" s="4"/>
       <c r="B270" s="1"/>
-      <c r="C270" s="22"/>
+      <c r="C270" s="15"/>
       <c r="D270" s="1"/>
       <c r="E270" s="1"/>
       <c r="F270" s="2"/>
@@ -6596,10 +6386,10 @@
       <c r="R270" s="3"/>
       <c r="S270" s="6"/>
     </row>
-    <row r="271" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A271" s="4"/>
       <c r="B271" s="1"/>
-      <c r="C271" s="22"/>
+      <c r="C271" s="15"/>
       <c r="D271" s="1"/>
       <c r="E271" s="1"/>
       <c r="F271" s="2"/>
@@ -6617,10 +6407,10 @@
       <c r="R271" s="3"/>
       <c r="S271" s="6"/>
     </row>
-    <row r="272" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A272" s="4"/>
       <c r="B272" s="1"/>
-      <c r="C272" s="22"/>
+      <c r="C272" s="15"/>
       <c r="D272" s="1"/>
       <c r="E272" s="1"/>
       <c r="F272" s="2"/>
@@ -6638,10 +6428,10 @@
       <c r="R272" s="3"/>
       <c r="S272" s="6"/>
     </row>
-    <row r="273" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A273" s="4"/>
       <c r="B273" s="1"/>
-      <c r="C273" s="22"/>
+      <c r="C273" s="15"/>
       <c r="D273" s="1"/>
       <c r="E273" s="1"/>
       <c r="F273" s="2"/>
@@ -6659,10 +6449,10 @@
       <c r="R273" s="3"/>
       <c r="S273" s="6"/>
     </row>
-    <row r="274" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A274" s="4"/>
       <c r="B274" s="1"/>
-      <c r="C274" s="22"/>
+      <c r="C274" s="15"/>
       <c r="D274" s="1"/>
       <c r="E274" s="1"/>
       <c r="F274" s="2"/>
@@ -6680,10 +6470,10 @@
       <c r="R274" s="3"/>
       <c r="S274" s="6"/>
     </row>
-    <row r="275" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A275" s="4"/>
       <c r="B275" s="1"/>
-      <c r="C275" s="22"/>
+      <c r="C275" s="15"/>
       <c r="D275" s="1"/>
       <c r="E275" s="1"/>
       <c r="F275" s="2"/>
@@ -6701,10 +6491,10 @@
       <c r="R275" s="3"/>
       <c r="S275" s="6"/>
     </row>
-    <row r="276" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A276" s="4"/>
       <c r="B276" s="1"/>
-      <c r="C276" s="22"/>
+      <c r="C276" s="15"/>
       <c r="D276" s="1"/>
       <c r="E276" s="1"/>
       <c r="F276" s="2"/>
@@ -6722,10 +6512,10 @@
       <c r="R276" s="3"/>
       <c r="S276" s="6"/>
     </row>
-    <row r="277" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A277" s="4"/>
       <c r="B277" s="1"/>
-      <c r="C277" s="22"/>
+      <c r="C277" s="15"/>
       <c r="D277" s="1"/>
       <c r="E277" s="1"/>
       <c r="F277" s="2"/>
@@ -6743,10 +6533,10 @@
       <c r="R277" s="3"/>
       <c r="S277" s="6"/>
     </row>
-    <row r="278" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A278" s="4"/>
       <c r="B278" s="1"/>
-      <c r="C278" s="22"/>
+      <c r="C278" s="15"/>
       <c r="D278" s="1"/>
       <c r="E278" s="1"/>
       <c r="F278" s="2"/>
@@ -6764,10 +6554,10 @@
       <c r="R278" s="3"/>
       <c r="S278" s="6"/>
     </row>
-    <row r="279" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A279" s="4"/>
       <c r="B279" s="1"/>
-      <c r="C279" s="22"/>
+      <c r="C279" s="15"/>
       <c r="D279" s="1"/>
       <c r="E279" s="1"/>
       <c r="F279" s="2"/>
@@ -6785,10 +6575,10 @@
       <c r="R279" s="3"/>
       <c r="S279" s="6"/>
     </row>
-    <row r="280" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A280" s="4"/>
       <c r="B280" s="1"/>
-      <c r="C280" s="22"/>
+      <c r="C280" s="15"/>
       <c r="D280" s="1"/>
       <c r="E280" s="1"/>
       <c r="F280" s="2"/>
@@ -6806,10 +6596,10 @@
       <c r="R280" s="3"/>
       <c r="S280" s="6"/>
     </row>
-    <row r="281" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A281" s="4"/>
       <c r="B281" s="1"/>
-      <c r="C281" s="22"/>
+      <c r="C281" s="15"/>
       <c r="D281" s="1"/>
       <c r="E281" s="1"/>
       <c r="F281" s="2"/>
@@ -6827,10 +6617,10 @@
       <c r="R281" s="3"/>
       <c r="S281" s="6"/>
     </row>
-    <row r="282" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A282" s="4"/>
       <c r="B282" s="1"/>
-      <c r="C282" s="22"/>
+      <c r="C282" s="15"/>
       <c r="D282" s="1"/>
       <c r="E282" s="1"/>
       <c r="F282" s="2"/>
@@ -6848,10 +6638,10 @@
       <c r="R282" s="3"/>
       <c r="S282" s="6"/>
     </row>
-    <row r="283" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A283" s="4"/>
       <c r="B283" s="1"/>
-      <c r="C283" s="22"/>
+      <c r="C283" s="15"/>
       <c r="D283" s="1"/>
       <c r="E283" s="1"/>
       <c r="F283" s="2"/>
@@ -6869,10 +6659,10 @@
       <c r="R283" s="3"/>
       <c r="S283" s="6"/>
     </row>
-    <row r="284" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A284" s="4"/>
       <c r="B284" s="1"/>
-      <c r="C284" s="22"/>
+      <c r="C284" s="15"/>
       <c r="D284" s="1"/>
       <c r="E284" s="1"/>
       <c r="F284" s="2"/>
@@ -6890,10 +6680,10 @@
       <c r="R284" s="3"/>
       <c r="S284" s="6"/>
     </row>
-    <row r="285" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A285" s="4"/>
       <c r="B285" s="1"/>
-      <c r="C285" s="22"/>
+      <c r="C285" s="15"/>
       <c r="D285" s="1"/>
       <c r="E285" s="1"/>
       <c r="F285" s="2"/>
@@ -6911,10 +6701,10 @@
       <c r="R285" s="3"/>
       <c r="S285" s="6"/>
     </row>
-    <row r="286" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A286" s="4"/>
       <c r="B286" s="1"/>
-      <c r="C286" s="22"/>
+      <c r="C286" s="15"/>
       <c r="D286" s="1"/>
       <c r="E286" s="1"/>
       <c r="F286" s="2"/>
@@ -6932,10 +6722,10 @@
       <c r="R286" s="3"/>
       <c r="S286" s="6"/>
     </row>
-    <row r="287" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A287" s="4"/>
       <c r="B287" s="1"/>
-      <c r="C287" s="22"/>
+      <c r="C287" s="15"/>
       <c r="D287" s="1"/>
       <c r="E287" s="1"/>
       <c r="F287" s="2"/>
@@ -6953,10 +6743,10 @@
       <c r="R287" s="3"/>
       <c r="S287" s="6"/>
     </row>
-    <row r="288" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A288" s="4"/>
       <c r="B288" s="1"/>
-      <c r="C288" s="22"/>
+      <c r="C288" s="15"/>
       <c r="D288" s="1"/>
       <c r="E288" s="1"/>
       <c r="F288" s="2"/>
@@ -6974,10 +6764,10 @@
       <c r="R288" s="3"/>
       <c r="S288" s="6"/>
     </row>
-    <row r="289" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A289" s="4"/>
       <c r="B289" s="1"/>
-      <c r="C289" s="22"/>
+      <c r="C289" s="15"/>
       <c r="D289" s="1"/>
       <c r="E289" s="1"/>
       <c r="F289" s="2"/>
@@ -6995,10 +6785,10 @@
       <c r="R289" s="3"/>
       <c r="S289" s="6"/>
     </row>
-    <row r="290" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A290" s="4"/>
       <c r="B290" s="1"/>
-      <c r="C290" s="22"/>
+      <c r="C290" s="15"/>
       <c r="D290" s="1"/>
       <c r="E290" s="1"/>
       <c r="F290" s="2"/>
@@ -7016,10 +6806,10 @@
       <c r="R290" s="3"/>
       <c r="S290" s="6"/>
     </row>
-    <row r="291" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A291" s="4"/>
       <c r="B291" s="1"/>
-      <c r="C291" s="22"/>
+      <c r="C291" s="15"/>
       <c r="D291" s="1"/>
       <c r="E291" s="1"/>
       <c r="F291" s="2"/>
@@ -7037,10 +6827,10 @@
       <c r="R291" s="3"/>
       <c r="S291" s="6"/>
     </row>
-    <row r="292" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A292" s="4"/>
       <c r="B292" s="1"/>
-      <c r="C292" s="22"/>
+      <c r="C292" s="15"/>
       <c r="D292" s="1"/>
       <c r="E292" s="1"/>
       <c r="F292" s="2"/>
@@ -7058,10 +6848,10 @@
       <c r="R292" s="3"/>
       <c r="S292" s="6"/>
     </row>
-    <row r="293" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A293" s="4"/>
       <c r="B293" s="1"/>
-      <c r="C293" s="22"/>
+      <c r="C293" s="15"/>
       <c r="D293" s="1"/>
       <c r="E293" s="1"/>
       <c r="F293" s="2"/>
@@ -7079,10 +6869,10 @@
       <c r="R293" s="3"/>
       <c r="S293" s="6"/>
     </row>
-    <row r="294" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A294" s="4"/>
       <c r="B294" s="1"/>
-      <c r="C294" s="22"/>
+      <c r="C294" s="15"/>
       <c r="D294" s="1"/>
       <c r="E294" s="1"/>
       <c r="F294" s="2"/>
@@ -7100,10 +6890,10 @@
       <c r="R294" s="3"/>
       <c r="S294" s="6"/>
     </row>
-    <row r="295" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A295" s="4"/>
       <c r="B295" s="1"/>
-      <c r="C295" s="22"/>
+      <c r="C295" s="15"/>
       <c r="D295" s="1"/>
       <c r="E295" s="1"/>
       <c r="F295" s="2"/>
@@ -7121,10 +6911,10 @@
       <c r="R295" s="3"/>
       <c r="S295" s="6"/>
     </row>
-    <row r="296" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A296" s="4"/>
       <c r="B296" s="1"/>
-      <c r="C296" s="22"/>
+      <c r="C296" s="15"/>
       <c r="D296" s="1"/>
       <c r="E296" s="1"/>
       <c r="F296" s="2"/>
@@ -7142,10 +6932,10 @@
       <c r="R296" s="3"/>
       <c r="S296" s="6"/>
     </row>
-    <row r="297" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A297" s="4"/>
       <c r="B297" s="1"/>
-      <c r="C297" s="22"/>
+      <c r="C297" s="15"/>
       <c r="D297" s="1"/>
       <c r="E297" s="1"/>
       <c r="F297" s="2"/>
@@ -7163,10 +6953,10 @@
       <c r="R297" s="3"/>
       <c r="S297" s="6"/>
     </row>
-    <row r="298" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A298" s="4"/>
       <c r="B298" s="1"/>
-      <c r="C298" s="22"/>
+      <c r="C298" s="15"/>
       <c r="D298" s="1"/>
       <c r="E298" s="1"/>
       <c r="F298" s="2"/>
@@ -7184,10 +6974,10 @@
       <c r="R298" s="3"/>
       <c r="S298" s="6"/>
     </row>
-    <row r="299" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A299" s="4"/>
       <c r="B299" s="1"/>
-      <c r="C299" s="22"/>
+      <c r="C299" s="15"/>
       <c r="D299" s="1"/>
       <c r="E299" s="1"/>
       <c r="F299" s="2"/>
@@ -7205,10 +6995,10 @@
       <c r="R299" s="3"/>
       <c r="S299" s="6"/>
     </row>
-    <row r="300" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A300" s="4"/>
       <c r="B300" s="1"/>
-      <c r="C300" s="22"/>
+      <c r="C300" s="15"/>
       <c r="D300" s="1"/>
       <c r="E300" s="1"/>
       <c r="F300" s="2"/>
@@ -7226,10 +7016,10 @@
       <c r="R300" s="3"/>
       <c r="S300" s="6"/>
     </row>
-    <row r="301" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A301" s="4"/>
       <c r="B301" s="1"/>
-      <c r="C301" s="22"/>
+      <c r="C301" s="15"/>
       <c r="D301" s="1"/>
       <c r="E301" s="1"/>
       <c r="F301" s="2"/>
@@ -7247,10 +7037,10 @@
       <c r="R301" s="3"/>
       <c r="S301" s="6"/>
     </row>
-    <row r="302" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A302" s="4"/>
       <c r="B302" s="1"/>
-      <c r="C302" s="22"/>
+      <c r="C302" s="15"/>
       <c r="D302" s="1"/>
       <c r="E302" s="1"/>
       <c r="F302" s="2"/>
@@ -7268,10 +7058,10 @@
       <c r="R302" s="3"/>
       <c r="S302" s="6"/>
     </row>
-    <row r="303" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A303" s="4"/>
       <c r="B303" s="1"/>
-      <c r="C303" s="22"/>
+      <c r="C303" s="15"/>
       <c r="D303" s="1"/>
       <c r="E303" s="1"/>
       <c r="F303" s="2"/>
@@ -7289,10 +7079,10 @@
       <c r="R303" s="3"/>
       <c r="S303" s="6"/>
     </row>
-    <row r="304" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A304" s="4"/>
       <c r="B304" s="1"/>
-      <c r="C304" s="22"/>
+      <c r="C304" s="15"/>
       <c r="D304" s="1"/>
       <c r="E304" s="1"/>
       <c r="F304" s="2"/>
@@ -7311,14 +7101,11 @@
       <c r="S304" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="1">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="H2:I2"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>